<commit_message>
Model: anchor FOB on real Canadian retail; add max-FOB-to-band column
Replaces arbitrary FOB placeholders with Organika's 2026 Canadian shelf
prices (Enhanced Collagen CAD29.99, Magnesium Bisglycinate CAD27.99,
Digest & Renew Greens CAD43.49, Whole Psyllium CAD25.99) times an
editable export-FOB ratio (40%, rule of thumb) on Controls. Probiotic
and vitamin C retail remain flagged placeholders (no clean SKU found).
Adds 'Max FOB to hit band midpoint (CAD)' per SKU by inverting the
margin stack. Finding: collagen lands below the VN premium band with
headroom; magnesium sits at the band ceiling; greens and fibre land
above band. 142 formulas, zero errors.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CHL2VrJ5edbBW6zFNsXfxt
</commit_message>
<xml_diff>
--- a/vietnam-margin-model.xlsx
+++ b/vietnam-margin-model.xlsx
@@ -138,6 +138,18 @@
         </r>
       </text>
     </comment>
+    <comment ref="B21" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Rule of thumb (LOW): brand wholesale ~50% of retail; export FOB at or below domestic wholesale. Replace with Organika export price list.</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
@@ -156,7 +168,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">PLACEHOLDER FOB. Replace with real Organika cost (CAD/unit).</t>
+          <t xml:space="preserve">Goodness Me / Voila CAD29.99; Well.ca CAD24.99 (2026, MEDIUM)</t>
         </r>
       </text>
     </comment>
@@ -168,7 +180,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">PLACEHOLDER FOB. Replace with real Organika cost (CAD/unit).</t>
+          <t xml:space="preserve">organika.com CAD27.99; Goodness Me CAD26.99 (2026, MEDIUM)</t>
         </r>
       </text>
     </comment>
@@ -180,7 +192,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">PLACEHOLDER FOB. Replace with real Organika cost (CAD/unit).</t>
+          <t xml:space="preserve">Well.ca CAD43.49 (2026, MEDIUM)</t>
         </r>
       </text>
     </comment>
@@ -192,7 +204,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">PLACEHOLDER FOB. Replace with real Organika cost (CAD/unit).</t>
+          <t xml:space="preserve">Well.ca CAD25.99 (2026, MEDIUM)</t>
         </r>
       </text>
     </comment>
@@ -204,7 +216,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">PLACEHOLDER FOB. Replace with real Organika cost (CAD/unit).</t>
+          <t xml:space="preserve">PLACEHOLDER: no adult Organika probiotic retail price found (Veggie Gummies w/ probiotic CAD45.97; baby drops CAD37.49)</t>
         </r>
       </text>
     </comment>
@@ -216,7 +228,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">PLACEHOLDER FOB. Replace with real Organika cost (CAD/unit).</t>
+          <t xml:space="preserve">PLACEHOLDER: no standalone Organika vitamin C SKU found; confirm the SKU exists</t>
         </r>
       </text>
     </comment>
@@ -307,7 +319,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="113">
   <si>
     <t xml:space="preserve">Organika — Vietnam Landed Cost &amp; Margin Model</t>
   </si>
@@ -327,7 +339,7 @@
     <t xml:space="preserve">2</t>
   </si>
   <si>
-    <t xml:space="preserve">On Landed Cost, replace the yellow FOB cells with real Organika FOB per unit (CAD). These are placeholders.</t>
+    <t xml:space="preserve">On Controls, set the export FOB ratio, or replace it with real export prices. LandedCost derives FOB from real Canadian retail.</t>
   </si>
   <si>
     <t xml:space="preserve">3</t>
@@ -417,7 +429,7 @@
     <t xml:space="preserve">FOB costs</t>
   </si>
   <si>
-    <t xml:space="preserve">PLACEHOLDERS. No real Organika COGS was available; replace before quoting.</t>
+    <t xml:space="preserve">ESTIMATED: Canadian retail (real 2026 shelf prices) x export FOB ratio (40%, rule of thumb) on Controls. Probiotic and vitamin C retail are placeholders. Replace with the Organika export price list.</t>
   </si>
   <si>
     <t xml:space="preserve">Controls — set once, drives every tab</t>
@@ -465,6 +477,12 @@
     <t xml:space="preserve">Units per SKU per year (amort base)</t>
   </si>
   <si>
+    <t xml:space="preserve">Export pricing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Export FOB as % of Canadian retail</t>
+  </si>
+  <si>
     <t xml:space="preserve">Landed cost per unit (CIF + duty), by SKU</t>
   </si>
   <si>
@@ -474,6 +492,9 @@
     <t xml:space="preserve">Role</t>
   </si>
   <si>
+    <t xml:space="preserve">Canadian retail (CAD)</t>
+  </si>
+  <si>
     <t xml:space="preserve">FOB (CAD)</t>
   </si>
   <si>
@@ -504,16 +525,16 @@
     <t xml:space="preserve">Credential flag</t>
   </si>
   <si>
-    <t xml:space="preserve">Magnesium bisglycinate</t>
+    <t xml:space="preserve">Magnesium bisglycinate (120 caps)</t>
   </si>
   <si>
     <t xml:space="preserve">Lead SKU</t>
   </si>
   <si>
-    <t xml:space="preserve">Greens / superfood</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fibre (psyllium/inulin)</t>
+    <t xml:space="preserve">Greens: Digest &amp; Renew (340g)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fibre: Whole Psyllium (454g)</t>
   </si>
   <si>
     <t xml:space="preserve">Range filler</t>
@@ -528,7 +549,7 @@
     <t xml:space="preserve">Vitamin C / dailies</t>
   </si>
   <si>
-    <t xml:space="preserve">FOB cells are placeholders (Controls legend). All other columns are formulas driven by Controls.</t>
+    <t xml:space="preserve">Canadian retail: real 2026 shelf prices (hover for source); yellow = placeholder. FOB = retail x export ratio on Controls (rule of thumb, replace with Organika export price list).</t>
   </si>
   <si>
     <t xml:space="preserve">SKU economics — shelf price vs the real Vietnamese shelf</t>
@@ -561,7 +582,7 @@
     <t xml:space="preserve">Position</t>
   </si>
   <si>
-    <t xml:space="preserve">Shelf (daily, for dailies)</t>
+    <t xml:space="preserve">Max FOB to hit band midpoint (CAD)</t>
   </si>
   <si>
     <t xml:space="preserve">Channel economics — what the brand nets per unit</t>
@@ -810,44 +831,40 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="27">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -855,47 +872,59 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="169" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="170" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -903,11 +932,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1166,175 +1195,175 @@
   <dimension ref="A1:B24"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="110"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="110"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4"/>
-      <c r="B3" s="4"/>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="5" t="s">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3"/>
+      <c r="B3" s="3"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="4"/>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
+      <c r="B4" s="3"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="3" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="3" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="3" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4"/>
-      <c r="B10" s="4"/>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="5" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="3"/>
+      <c r="B10" s="3"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B11" s="4"/>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="6" t="s">
+      <c r="B11" s="3"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="7" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="3" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="7" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="B14" s="3" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="7" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="3" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4"/>
-      <c r="B16" s="4"/>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="5" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="3"/>
+      <c r="B16" s="3"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B17" s="4"/>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="7" t="s">
+      <c r="B17" s="3"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="B18" s="4" t="s">
+      <c r="B18" s="3" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="7" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="B19" s="4" t="s">
+      <c r="B19" s="3" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="7" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="B20" s="4" t="s">
+      <c r="B20" s="3" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="7" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="B21" s="4" t="s">
+      <c r="B21" s="3" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="7" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="B22" s="3" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="7" t="s">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="B23" s="4" t="s">
+      <c r="B23" s="3" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="7" t="s">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="B24" s="4" t="s">
+      <c r="B24" s="3" t="s">
         <v>36</v>
       </c>
     </row>
@@ -1354,134 +1383,150 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="5" t="s">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="4" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="7" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="B4" s="8" t="n">
+      <c r="B4" s="7" t="n">
         <v>18450</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="2" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="7" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="B5" s="8" t="n">
+      <c r="B5" s="7" t="n">
         <v>26200</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="2" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="7" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="B8" s="8" t="n">
+      <c r="B8" s="7" t="n">
         <v>11800</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" s="2" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="7" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="B9" s="9" t="n">
+      <c r="B9" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="D9" s="2" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="B10" s="9" t="n">
+      <c r="B10" s="8" t="n">
         <v>0.08</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="D10" s="2" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="5" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="7" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="B13" s="9" t="n">
+      <c r="B13" s="8" t="n">
         <v>0.45</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="D13" s="2" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="7" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="B14" s="9" t="n">
+      <c r="B14" s="8" t="n">
         <v>0.3</v>
       </c>
-      <c r="D14" s="3" t="s">
+      <c r="D14" s="2" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="5" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="7" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="B17" s="8" t="n">
+      <c r="B17" s="7" t="n">
         <v>70000000</v>
       </c>
-      <c r="D17" s="3" t="s">
+      <c r="D17" s="2" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="7" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="B18" s="8" t="n">
+      <c r="B18" s="7" t="n">
         <v>20000</v>
       </c>
-      <c r="D18" s="3" t="s">
+      <c r="D18" s="2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="B21" s="8" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="D21" s="2" t="s">
         <v>40</v>
       </c>
     </row>
@@ -1502,292 +1547,320 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="4" style="1" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="1" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="5" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="15"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="10" t="s">
-        <v>53</v>
-      </c>
-      <c r="B3" s="10" t="s">
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="C3" s="10" t="s">
+    </row>
+    <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="D3" s="10" t="s">
+      <c r="B3" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="E3" s="10" t="s">
+      <c r="C3" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="F3" s="10" t="s">
+      <c r="D3" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="G3" s="10" t="s">
+      <c r="E3" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="H3" s="10" t="s">
+      <c r="F3" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="I3" s="10" t="s">
+      <c r="G3" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="J3" s="10" t="s">
+      <c r="H3" s="9" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="7" t="s">
+      <c r="I3" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="J3" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="C4" s="11" t="n">
-        <v>12</v>
-      </c>
-      <c r="D4" s="12" t="n">
-        <f aca="false">C4*Controls!$B$4</f>
-        <v>221400</v>
-      </c>
-      <c r="E4" s="13" t="n">
+      <c r="K3" s="9" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="C4" s="10" t="n">
+        <v>29.99</v>
+      </c>
+      <c r="D4" s="11" t="n">
+        <f aca="false">C4*Controls!$B$21</f>
+        <v>11.996</v>
+      </c>
+      <c r="E4" s="12" t="n">
+        <f aca="false">D4*Controls!$B$4</f>
+        <v>221326.2</v>
+      </c>
+      <c r="F4" s="13" t="n">
         <f aca="false">Controls!$B$8</f>
         <v>11800</v>
       </c>
-      <c r="F4" s="13" t="n">
-        <f aca="false">D4+E4</f>
-        <v>233200</v>
-      </c>
-      <c r="G4" s="13" t="n">
-        <f aca="false">F4*Controls!$B$9</f>
+      <c r="G4" s="12" t="n">
+        <f aca="false">E4+F4</f>
+        <v>233126.2</v>
+      </c>
+      <c r="H4" s="12" t="n">
+        <f aca="false">G4*Controls!$B$9</f>
         <v>0</v>
       </c>
-      <c r="H4" s="13" t="n">
-        <f aca="false">F4+G4</f>
-        <v>233200</v>
-      </c>
-      <c r="I4" s="13" t="n">
+      <c r="I4" s="12" t="n">
+        <f aca="false">G4+H4</f>
+        <v>233126.2</v>
+      </c>
+      <c r="J4" s="13" t="n">
         <f aca="false">Controls!$B$17/Controls!$B$18</f>
         <v>3500</v>
       </c>
-      <c r="J4" s="13" t="n">
-        <f aca="false">H4+I4</f>
-        <v>236700</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="C5" s="11" t="n">
-        <v>6</v>
-      </c>
-      <c r="D5" s="12" t="n">
-        <f aca="false">C5*Controls!$B$4</f>
-        <v>110700</v>
-      </c>
-      <c r="E5" s="13" t="n">
+      <c r="K4" s="12" t="n">
+        <f aca="false">I4+J4</f>
+        <v>236626.2</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C5" s="10" t="n">
+        <v>27.99</v>
+      </c>
+      <c r="D5" s="11" t="n">
+        <f aca="false">C5*Controls!$B$21</f>
+        <v>11.196</v>
+      </c>
+      <c r="E5" s="12" t="n">
+        <f aca="false">D5*Controls!$B$4</f>
+        <v>206566.2</v>
+      </c>
+      <c r="F5" s="13" t="n">
         <f aca="false">Controls!$B$8</f>
         <v>11800</v>
       </c>
-      <c r="F5" s="13" t="n">
-        <f aca="false">D5+E5</f>
-        <v>122500</v>
-      </c>
-      <c r="G5" s="13" t="n">
-        <f aca="false">F5*Controls!$B$9</f>
+      <c r="G5" s="12" t="n">
+        <f aca="false">E5+F5</f>
+        <v>218366.2</v>
+      </c>
+      <c r="H5" s="12" t="n">
+        <f aca="false">G5*Controls!$B$9</f>
         <v>0</v>
       </c>
-      <c r="H5" s="13" t="n">
-        <f aca="false">F5+G5</f>
-        <v>122500</v>
-      </c>
-      <c r="I5" s="13" t="n">
+      <c r="I5" s="12" t="n">
+        <f aca="false">G5+H5</f>
+        <v>218366.2</v>
+      </c>
+      <c r="J5" s="13" t="n">
         <f aca="false">Controls!$B$17/Controls!$B$18</f>
         <v>3500</v>
       </c>
-      <c r="J5" s="13" t="n">
-        <f aca="false">H5+I5</f>
-        <v>126000</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="C6" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="D6" s="12" t="n">
-        <f aca="false">C6*Controls!$B$4</f>
-        <v>147600</v>
-      </c>
-      <c r="E6" s="13" t="n">
+      <c r="K5" s="12" t="n">
+        <f aca="false">I5+J5</f>
+        <v>221866.2</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C6" s="10" t="n">
+        <v>43.49</v>
+      </c>
+      <c r="D6" s="11" t="n">
+        <f aca="false">C6*Controls!$B$21</f>
+        <v>17.396</v>
+      </c>
+      <c r="E6" s="12" t="n">
+        <f aca="false">D6*Controls!$B$4</f>
+        <v>320956.2</v>
+      </c>
+      <c r="F6" s="13" t="n">
         <f aca="false">Controls!$B$8</f>
         <v>11800</v>
       </c>
-      <c r="F6" s="13" t="n">
-        <f aca="false">D6+E6</f>
-        <v>159400</v>
-      </c>
-      <c r="G6" s="13" t="n">
-        <f aca="false">F6*Controls!$B$9</f>
+      <c r="G6" s="12" t="n">
+        <f aca="false">E6+F6</f>
+        <v>332756.2</v>
+      </c>
+      <c r="H6" s="12" t="n">
+        <f aca="false">G6*Controls!$B$9</f>
         <v>0</v>
       </c>
-      <c r="H6" s="13" t="n">
-        <f aca="false">F6+G6</f>
-        <v>159400</v>
-      </c>
-      <c r="I6" s="13" t="n">
+      <c r="I6" s="12" t="n">
+        <f aca="false">G6+H6</f>
+        <v>332756.2</v>
+      </c>
+      <c r="J6" s="13" t="n">
         <f aca="false">Controls!$B$17/Controls!$B$18</f>
         <v>3500</v>
       </c>
-      <c r="J6" s="13" t="n">
-        <f aca="false">H6+I6</f>
-        <v>162900</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="C7" s="11" t="n">
-        <v>5</v>
-      </c>
-      <c r="D7" s="12" t="n">
-        <f aca="false">C7*Controls!$B$4</f>
-        <v>92250</v>
-      </c>
-      <c r="E7" s="13" t="n">
+      <c r="K6" s="12" t="n">
+        <f aca="false">I6+J6</f>
+        <v>336256.2</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="C7" s="10" t="n">
+        <v>25.99</v>
+      </c>
+      <c r="D7" s="11" t="n">
+        <f aca="false">C7*Controls!$B$21</f>
+        <v>10.396</v>
+      </c>
+      <c r="E7" s="12" t="n">
+        <f aca="false">D7*Controls!$B$4</f>
+        <v>191806.2</v>
+      </c>
+      <c r="F7" s="13" t="n">
         <f aca="false">Controls!$B$8</f>
         <v>11800</v>
       </c>
-      <c r="F7" s="13" t="n">
-        <f aca="false">D7+E7</f>
-        <v>104050</v>
-      </c>
-      <c r="G7" s="13" t="n">
-        <f aca="false">F7*Controls!$B$9</f>
+      <c r="G7" s="12" t="n">
+        <f aca="false">E7+F7</f>
+        <v>203606.2</v>
+      </c>
+      <c r="H7" s="12" t="n">
+        <f aca="false">G7*Controls!$B$9</f>
         <v>0</v>
       </c>
-      <c r="H7" s="13" t="n">
-        <f aca="false">F7+G7</f>
-        <v>104050</v>
-      </c>
-      <c r="I7" s="13" t="n">
+      <c r="I7" s="12" t="n">
+        <f aca="false">G7+H7</f>
+        <v>203606.2</v>
+      </c>
+      <c r="J7" s="13" t="n">
         <f aca="false">Controls!$B$17/Controls!$B$18</f>
         <v>3500</v>
       </c>
-      <c r="J7" s="13" t="n">
-        <f aca="false">H7+I7</f>
-        <v>107550</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="7" t="s">
-        <v>70</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="C8" s="11" t="n">
-        <v>7</v>
-      </c>
-      <c r="D8" s="12" t="n">
-        <f aca="false">C8*Controls!$B$4</f>
-        <v>129150</v>
-      </c>
-      <c r="E8" s="13" t="n">
+      <c r="K7" s="12" t="n">
+        <f aca="false">I7+J7</f>
+        <v>207106.2</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="C8" s="14" t="n">
+        <v>35</v>
+      </c>
+      <c r="D8" s="11" t="n">
+        <f aca="false">C8*Controls!$B$21</f>
+        <v>14</v>
+      </c>
+      <c r="E8" s="12" t="n">
+        <f aca="false">D8*Controls!$B$4</f>
+        <v>258300</v>
+      </c>
+      <c r="F8" s="13" t="n">
         <f aca="false">Controls!$B$8</f>
         <v>11800</v>
       </c>
-      <c r="F8" s="13" t="n">
-        <f aca="false">D8+E8</f>
-        <v>140950</v>
-      </c>
-      <c r="G8" s="13" t="n">
-        <f aca="false">F8*Controls!$B$9</f>
+      <c r="G8" s="12" t="n">
+        <f aca="false">E8+F8</f>
+        <v>270100</v>
+      </c>
+      <c r="H8" s="12" t="n">
+        <f aca="false">G8*Controls!$B$9</f>
         <v>0</v>
       </c>
-      <c r="H8" s="13" t="n">
-        <f aca="false">F8+G8</f>
-        <v>140950</v>
-      </c>
-      <c r="I8" s="13" t="n">
+      <c r="I8" s="12" t="n">
+        <f aca="false">G8+H8</f>
+        <v>270100</v>
+      </c>
+      <c r="J8" s="13" t="n">
         <f aca="false">Controls!$B$17/Controls!$B$18</f>
         <v>3500</v>
       </c>
-      <c r="J8" s="13" t="n">
-        <f aca="false">H8+I8</f>
-        <v>144450</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="7" t="s">
+      <c r="K8" s="12" t="n">
+        <f aca="false">I8+J8</f>
+        <v>273600</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="B9" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="B9" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="C9" s="11" t="n">
-        <v>3</v>
-      </c>
-      <c r="D9" s="12" t="n">
-        <f aca="false">C9*Controls!$B$4</f>
-        <v>55350</v>
-      </c>
-      <c r="E9" s="13" t="n">
+      <c r="C9" s="14" t="n">
+        <v>15</v>
+      </c>
+      <c r="D9" s="11" t="n">
+        <f aca="false">C9*Controls!$B$21</f>
+        <v>6</v>
+      </c>
+      <c r="E9" s="12" t="n">
+        <f aca="false">D9*Controls!$B$4</f>
+        <v>110700</v>
+      </c>
+      <c r="F9" s="13" t="n">
         <f aca="false">Controls!$B$8</f>
         <v>11800</v>
       </c>
-      <c r="F9" s="13" t="n">
-        <f aca="false">D9+E9</f>
-        <v>67150</v>
-      </c>
-      <c r="G9" s="13" t="n">
-        <f aca="false">F9*Controls!$B$9</f>
+      <c r="G9" s="12" t="n">
+        <f aca="false">E9+F9</f>
+        <v>122500</v>
+      </c>
+      <c r="H9" s="12" t="n">
+        <f aca="false">G9*Controls!$B$9</f>
         <v>0</v>
       </c>
-      <c r="H9" s="13" t="n">
-        <f aca="false">F9+G9</f>
-        <v>67150</v>
-      </c>
-      <c r="I9" s="13" t="n">
+      <c r="I9" s="12" t="n">
+        <f aca="false">G9+H9</f>
+        <v>122500</v>
+      </c>
+      <c r="J9" s="13" t="n">
         <f aca="false">Controls!$B$17/Controls!$B$18</f>
         <v>3500</v>
       </c>
-      <c r="J9" s="13" t="n">
-        <f aca="false">H9+I9</f>
-        <v>70650</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="s">
-        <v>73</v>
+      <c r="K9" s="12" t="n">
+        <f aca="false">I9+J9</f>
+        <v>126000</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="2" t="s">
+        <v>76</v>
       </c>
     </row>
   </sheetData>
@@ -1810,340 +1883,340 @@
   <dimension ref="A1:L9"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="6" style="1" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="1" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="6" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="16"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="10" t="s">
-        <v>53</v>
-      </c>
-      <c r="B3" s="10" t="s">
-        <v>62</v>
-      </c>
-      <c r="C3" s="10" t="s">
-        <v>75</v>
-      </c>
-      <c r="D3" s="10" t="s">
-        <v>76</v>
-      </c>
-      <c r="E3" s="10" t="s">
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="F3" s="10" t="s">
+    </row>
+    <row r="3" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="C3" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="G3" s="10" t="s">
+      <c r="D3" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="H3" s="10" t="s">
+      <c r="E3" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="I3" s="10" t="s">
+      <c r="F3" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="J3" s="10" t="s">
+      <c r="G3" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="K3" s="10" t="s">
+      <c r="H3" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="L3" s="10" t="s">
+      <c r="I3" s="9" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="7" t="s">
-        <v>63</v>
-      </c>
-      <c r="B4" s="12" t="n">
-        <f aca="false">LandedCost!J4</f>
-        <v>236700</v>
-      </c>
-      <c r="C4" s="13" t="n">
+      <c r="J3" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="K3" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="L3" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="B4" s="13" t="n">
+        <f aca="false">LandedCost!K4</f>
+        <v>236626.2</v>
+      </c>
+      <c r="C4" s="12" t="n">
         <f aca="false">B4*(1+Controls!$B$13)</f>
-        <v>343215</v>
-      </c>
-      <c r="D4" s="13" t="n">
+        <v>343107.99</v>
+      </c>
+      <c r="D4" s="12" t="n">
         <f aca="false">C4/(1-Controls!$B$14)</f>
-        <v>490307.142857143</v>
-      </c>
-      <c r="E4" s="13" t="n">
+        <v>490154.271428571</v>
+      </c>
+      <c r="E4" s="12" t="n">
         <f aca="false">D4*(1+Controls!$B$10)</f>
-        <v>529531.714285714</v>
-      </c>
-      <c r="F4" s="14" t="n">
+        <v>529366.613142857</v>
+      </c>
+      <c r="F4" s="15" t="n">
         <f aca="false">E4/Controls!$B$5</f>
-        <v>20.2111341330425</v>
-      </c>
-      <c r="G4" s="15" t="n">
+        <v>20.2048325627045</v>
+      </c>
+      <c r="G4" s="16" t="n">
         <f aca="false">E4/Controls!$B$4</f>
-        <v>28.700905923345</v>
-      </c>
-      <c r="H4" s="16" t="n">
-        <f aca="false">E4/LandedCost!D4</f>
-        <v>2.39174216027875</v>
-      </c>
-      <c r="I4" s="17" t="n">
+        <v>28.6919573519164</v>
+      </c>
+      <c r="H4" s="17" t="n">
+        <f aca="false">E4/LandedCost!E4</f>
+        <v>2.39179371056322</v>
+      </c>
+      <c r="I4" s="18" t="n">
         <v>650000</v>
       </c>
-      <c r="J4" s="17" t="n">
+      <c r="J4" s="18" t="n">
         <v>850000</v>
       </c>
-      <c r="K4" s="18" t="str">
+      <c r="K4" s="19" t="str">
         <f aca="false">IF(E4&lt;I4,"Below band — room to price up",IF(E4&gt;J4,"Above band — promo-room risk","Within band"))</f>
         <v>Below band — room to price up</v>
       </c>
-      <c r="L4" s="13" t="n">
-        <f aca="false">E4/30</f>
-        <v>17651.0571428571</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="B5" s="12" t="n">
-        <f aca="false">LandedCost!J5</f>
-        <v>126000</v>
-      </c>
-      <c r="C5" s="13" t="n">
+      <c r="L4" s="20" t="n">
+        <f aca="false">(((I4+J4)/2/((1+Controls!$B$13)/(1-Controls!$B$14)*(1+Controls!$B$10))-Controls!$B$17/Controls!$B$18)/(1+Controls!$B$9)-Controls!$B$8)/Controls!$B$4</f>
+        <v>17.3414114984062</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="B5" s="13" t="n">
+        <f aca="false">LandedCost!K5</f>
+        <v>221866.2</v>
+      </c>
+      <c r="C5" s="12" t="n">
         <f aca="false">B5*(1+Controls!$B$13)</f>
-        <v>182700</v>
-      </c>
-      <c r="D5" s="13" t="n">
+        <v>321705.99</v>
+      </c>
+      <c r="D5" s="12" t="n">
         <f aca="false">C5/(1-Controls!$B$14)</f>
-        <v>261000</v>
-      </c>
-      <c r="E5" s="13" t="n">
+        <v>459579.985714286</v>
+      </c>
+      <c r="E5" s="12" t="n">
         <f aca="false">D5*(1+Controls!$B$10)</f>
-        <v>281880</v>
-      </c>
-      <c r="F5" s="14" t="n">
+        <v>496346.384571429</v>
+      </c>
+      <c r="F5" s="15" t="n">
         <f aca="false">E5/Controls!$B$5</f>
-        <v>10.7587786259542</v>
-      </c>
-      <c r="G5" s="15" t="n">
+        <v>18.9445184950927</v>
+      </c>
+      <c r="G5" s="16" t="n">
         <f aca="false">E5/Controls!$B$4</f>
-        <v>15.2780487804878</v>
-      </c>
-      <c r="H5" s="16" t="n">
-        <f aca="false">E5/LandedCost!D5</f>
-        <v>2.54634146341463</v>
-      </c>
-      <c r="I5" s="17" t="n">
+        <v>26.9022430662021</v>
+      </c>
+      <c r="H5" s="17" t="n">
+        <f aca="false">E5/LandedCost!E5</f>
+        <v>2.40284414667757</v>
+      </c>
+      <c r="I5" s="18" t="n">
         <v>220000</v>
       </c>
-      <c r="J5" s="17" t="n">
+      <c r="J5" s="18" t="n">
         <v>500000</v>
       </c>
-      <c r="K5" s="18" t="str">
+      <c r="K5" s="19" t="str">
         <f aca="false">IF(E5&lt;I5,"Below band — room to price up",IF(E5&gt;J5,"Above band — promo-room risk","Within band"))</f>
         <v>Within band</v>
       </c>
-      <c r="L5" s="13" t="n">
-        <f aca="false">E5/30</f>
-        <v>9396</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="B6" s="12" t="n">
-        <f aca="false">LandedCost!J6</f>
-        <v>162900</v>
-      </c>
-      <c r="C6" s="13" t="n">
+      <c r="L5" s="20" t="n">
+        <f aca="false">(((I5+J5)/2/((1+Controls!$B$13)/(1-Controls!$B$14)*(1+Controls!$B$10))-Controls!$B$17/Controls!$B$18)/(1+Controls!$B$9)-Controls!$B$8)/Controls!$B$4</f>
+        <v>7.89265800703984</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="B6" s="13" t="n">
+        <f aca="false">LandedCost!K6</f>
+        <v>336256.2</v>
+      </c>
+      <c r="C6" s="12" t="n">
         <f aca="false">B6*(1+Controls!$B$13)</f>
-        <v>236205</v>
-      </c>
-      <c r="D6" s="13" t="n">
+        <v>487571.49</v>
+      </c>
+      <c r="D6" s="12" t="n">
         <f aca="false">C6/(1-Controls!$B$14)</f>
-        <v>337435.714285714</v>
-      </c>
-      <c r="E6" s="13" t="n">
+        <v>696530.7</v>
+      </c>
+      <c r="E6" s="12" t="n">
         <f aca="false">D6*(1+Controls!$B$10)</f>
-        <v>364430.571428572</v>
-      </c>
-      <c r="F6" s="14" t="n">
+        <v>752253.156</v>
+      </c>
+      <c r="F6" s="15" t="n">
         <f aca="false">E6/Controls!$B$5</f>
-        <v>13.9095637949836</v>
-      </c>
-      <c r="G6" s="15" t="n">
+        <v>28.711952519084</v>
+      </c>
+      <c r="G6" s="16" t="n">
         <f aca="false">E6/Controls!$B$4</f>
-        <v>19.7523344947735</v>
-      </c>
-      <c r="H6" s="16" t="n">
-        <f aca="false">E6/LandedCost!D6</f>
-        <v>2.46904181184669</v>
-      </c>
-      <c r="I6" s="17" t="n">
+        <v>40.7725287804878</v>
+      </c>
+      <c r="H6" s="17" t="n">
+        <f aca="false">E6/LandedCost!E6</f>
+        <v>2.34378758223085</v>
+      </c>
+      <c r="I6" s="18" t="n">
         <v>350000</v>
       </c>
-      <c r="J6" s="17" t="n">
+      <c r="J6" s="18" t="n">
         <v>600000</v>
       </c>
-      <c r="K6" s="18" t="str">
+      <c r="K6" s="19" t="str">
         <f aca="false">IF(E6&lt;I6,"Below band — room to price up",IF(E6&gt;J6,"Above band — promo-room risk","Within band"))</f>
-        <v>Within band</v>
-      </c>
-      <c r="L6" s="13" t="n">
-        <f aca="false">E6/30</f>
-        <v>12147.6857142857</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="B7" s="12" t="n">
-        <f aca="false">LandedCost!J7</f>
-        <v>107550</v>
-      </c>
-      <c r="C7" s="13" t="n">
+        <v>Above band — promo-room risk</v>
+      </c>
+      <c r="L6" s="20" t="n">
+        <f aca="false">(((I6+J6)/2/((1+Controls!$B$13)/(1-Controls!$B$14)*(1+Controls!$B$10))-Controls!$B$17/Controls!$B$18)/(1+Controls!$B$9)-Controls!$B$8)/Controls!$B$4</f>
+        <v>10.6788289083402</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="B7" s="13" t="n">
+        <f aca="false">LandedCost!K7</f>
+        <v>207106.2</v>
+      </c>
+      <c r="C7" s="12" t="n">
         <f aca="false">B7*(1+Controls!$B$13)</f>
-        <v>155947.5</v>
-      </c>
-      <c r="D7" s="13" t="n">
+        <v>300303.99</v>
+      </c>
+      <c r="D7" s="12" t="n">
         <f aca="false">C7/(1-Controls!$B$14)</f>
-        <v>222782.142857143</v>
-      </c>
-      <c r="E7" s="13" t="n">
+        <v>429005.7</v>
+      </c>
+      <c r="E7" s="12" t="n">
         <f aca="false">D7*(1+Controls!$B$10)</f>
-        <v>240604.714285714</v>
-      </c>
-      <c r="F7" s="14" t="n">
+        <v>463326.156</v>
+      </c>
+      <c r="F7" s="15" t="n">
         <f aca="false">E7/Controls!$B$5</f>
-        <v>9.18338604143948</v>
-      </c>
-      <c r="G7" s="15" t="n">
+        <v>17.6842044274809</v>
+      </c>
+      <c r="G7" s="16" t="n">
         <f aca="false">E7/Controls!$B$4</f>
-        <v>13.040905923345</v>
-      </c>
-      <c r="H7" s="16" t="n">
-        <f aca="false">E7/LandedCost!D7</f>
-        <v>2.60818118466899</v>
-      </c>
-      <c r="I7" s="17" t="n">
+        <v>25.1125287804878</v>
+      </c>
+      <c r="H7" s="17" t="n">
+        <f aca="false">E7/LandedCost!E7</f>
+        <v>2.41559530400999</v>
+      </c>
+      <c r="I7" s="18" t="n">
         <v>250000</v>
       </c>
-      <c r="J7" s="17" t="n">
+      <c r="J7" s="18" t="n">
         <v>400000</v>
       </c>
-      <c r="K7" s="18" t="str">
+      <c r="K7" s="19" t="str">
         <f aca="false">IF(E7&lt;I7,"Below band — room to price up",IF(E7&gt;J7,"Above band — promo-room risk","Within band"))</f>
-        <v>Below band — room to price up</v>
-      </c>
-      <c r="L7" s="13" t="n">
-        <f aca="false">E7/30</f>
-        <v>8020.15714285714</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="7" t="s">
-        <v>70</v>
-      </c>
-      <c r="B8" s="12" t="n">
-        <f aca="false">LandedCost!J8</f>
-        <v>144450</v>
-      </c>
-      <c r="C8" s="13" t="n">
+        <v>Above band — promo-room risk</v>
+      </c>
+      <c r="L7" s="20" t="n">
+        <f aca="false">(((I7+J7)/2/((1+Controls!$B$13)/(1-Controls!$B$14)*(1+Controls!$B$10))-Controls!$B$17/Controls!$B$18)/(1+Controls!$B$9)-Controls!$B$8)/Controls!$B$4</f>
+        <v>7.04469295012235</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="B8" s="13" t="n">
+        <f aca="false">LandedCost!K8</f>
+        <v>273600</v>
+      </c>
+      <c r="C8" s="12" t="n">
         <f aca="false">B8*(1+Controls!$B$13)</f>
-        <v>209452.5</v>
-      </c>
-      <c r="D8" s="13" t="n">
+        <v>396720</v>
+      </c>
+      <c r="D8" s="12" t="n">
         <f aca="false">C8/(1-Controls!$B$14)</f>
-        <v>299217.857142857</v>
-      </c>
-      <c r="E8" s="13" t="n">
+        <v>566742.857142857</v>
+      </c>
+      <c r="E8" s="12" t="n">
         <f aca="false">D8*(1+Controls!$B$10)</f>
-        <v>323155.285714286</v>
-      </c>
-      <c r="F8" s="14" t="n">
+        <v>612082.285714286</v>
+      </c>
+      <c r="F8" s="15" t="n">
         <f aca="false">E8/Controls!$B$5</f>
-        <v>12.3341712104689</v>
-      </c>
-      <c r="G8" s="15" t="n">
+        <v>23.361919302072</v>
+      </c>
+      <c r="G8" s="16" t="n">
         <f aca="false">E8/Controls!$B$4</f>
-        <v>17.5151916376307</v>
-      </c>
-      <c r="H8" s="16" t="n">
-        <f aca="false">E8/LandedCost!D8</f>
-        <v>2.50217023394724</v>
-      </c>
-      <c r="I8" s="17" t="n">
+        <v>33.1751916376307</v>
+      </c>
+      <c r="H8" s="17" t="n">
+        <f aca="false">E8/LandedCost!E8</f>
+        <v>2.36965654554505</v>
+      </c>
+      <c r="I8" s="18" t="n">
         <v>350000</v>
       </c>
-      <c r="J8" s="17" t="n">
+      <c r="J8" s="18" t="n">
         <v>550000</v>
       </c>
-      <c r="K8" s="18" t="str">
+      <c r="K8" s="19" t="str">
         <f aca="false">IF(E8&lt;I8,"Below band — room to price up",IF(E8&gt;J8,"Above band — promo-room risk","Within band"))</f>
-        <v>Below band — room to price up</v>
-      </c>
-      <c r="L8" s="13" t="n">
-        <f aca="false">E8/30</f>
-        <v>10771.8428571429</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="B9" s="12" t="n">
-        <f aca="false">LandedCost!J9</f>
-        <v>70650</v>
-      </c>
-      <c r="C9" s="13" t="n">
+        <v>Above band — promo-room risk</v>
+      </c>
+      <c r="L8" s="20" t="n">
+        <f aca="false">(((I8+J8)/2/((1+Controls!$B$13)/(1-Controls!$B$14)*(1+Controls!$B$10))-Controls!$B$17/Controls!$B$18)/(1+Controls!$B$9)-Controls!$B$8)/Controls!$B$4</f>
+        <v>10.0731395819705</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="B9" s="13" t="n">
+        <f aca="false">LandedCost!K9</f>
+        <v>126000</v>
+      </c>
+      <c r="C9" s="12" t="n">
         <f aca="false">B9*(1+Controls!$B$13)</f>
-        <v>102442.5</v>
-      </c>
-      <c r="D9" s="13" t="n">
+        <v>182700</v>
+      </c>
+      <c r="D9" s="12" t="n">
         <f aca="false">C9/(1-Controls!$B$14)</f>
-        <v>146346.428571429</v>
-      </c>
-      <c r="E9" s="13" t="n">
+        <v>261000</v>
+      </c>
+      <c r="E9" s="12" t="n">
         <f aca="false">D9*(1+Controls!$B$10)</f>
-        <v>158054.142857143</v>
-      </c>
-      <c r="F9" s="14" t="n">
+        <v>281880</v>
+      </c>
+      <c r="F9" s="15" t="n">
         <f aca="false">E9/Controls!$B$5</f>
-        <v>6.03260087241003</v>
-      </c>
-      <c r="G9" s="15" t="n">
+        <v>10.7587786259542</v>
+      </c>
+      <c r="G9" s="16" t="n">
         <f aca="false">E9/Controls!$B$4</f>
-        <v>8.56662020905923</v>
-      </c>
-      <c r="H9" s="16" t="n">
-        <f aca="false">E9/LandedCost!D9</f>
-        <v>2.85554006968641</v>
-      </c>
-      <c r="I9" s="17" t="n">
+        <v>15.2780487804878</v>
+      </c>
+      <c r="H9" s="17" t="n">
+        <f aca="false">E9/LandedCost!E9</f>
+        <v>2.54634146341463</v>
+      </c>
+      <c r="I9" s="18" t="n">
         <v>60000</v>
       </c>
-      <c r="J9" s="17" t="n">
+      <c r="J9" s="18" t="n">
         <v>150000</v>
       </c>
-      <c r="K9" s="18" t="str">
+      <c r="K9" s="19" t="str">
         <f aca="false">IF(E9&lt;I9,"Below band — room to price up",IF(E9&gt;J9,"Above band — promo-room risk","Within band"))</f>
         <v>Above band — promo-room risk</v>
       </c>
-      <c r="L9" s="13" t="n">
-        <f aca="false">E9/30</f>
-        <v>5268.47142857143</v>
+      <c r="L9" s="20" t="n">
+        <f aca="false">(((I9+J9)/2/((1+Controls!$B$13)/(1-Controls!$B$14)*(1+Controls!$B$10))-Controls!$B$17/Controls!$B$18)/(1+Controls!$B$9)-Controls!$B$8)/Controls!$B$4</f>
+        <v>1.71462687806955</v>
       </c>
     </row>
   </sheetData>
@@ -2166,181 +2239,181 @@
   <dimension ref="A1:H12"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="4" style="1" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="4" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="12"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="7" t="s">
-        <v>87</v>
-      </c>
-      <c r="B4" s="19" t="n">
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="B4" s="21" t="n">
         <f aca="false">SKU_Economics!E4</f>
-        <v>529531.714285714</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="10" t="s">
-        <v>88</v>
-      </c>
-      <c r="B6" s="10" t="s">
-        <v>89</v>
-      </c>
-      <c r="C6" s="10" t="s">
-        <v>90</v>
-      </c>
-      <c r="D6" s="10" t="s">
+        <v>529366.613142857</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="E6" s="10" t="s">
+      <c r="B6" s="9" t="s">
         <v>92</v>
       </c>
-      <c r="F6" s="10" t="s">
+      <c r="C6" s="9" t="s">
         <v>93</v>
       </c>
-      <c r="G6" s="10" t="s">
+      <c r="D6" s="9" t="s">
         <v>94</v>
       </c>
-      <c r="H6" s="10" t="s">
+      <c r="E6" s="9" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="7" t="s">
+      <c r="F6" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="B7" s="9" t="n">
+      <c r="G6" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="H6" s="9" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="B7" s="8" t="n">
         <v>0.21</v>
       </c>
-      <c r="C7" s="9" t="n">
+      <c r="C7" s="8" t="n">
         <v>0.15</v>
       </c>
-      <c r="D7" s="9" t="n">
+      <c r="D7" s="8" t="n">
         <v>0.07</v>
       </c>
-      <c r="E7" s="20" t="n">
+      <c r="E7" s="22" t="n">
         <f aca="false">B7+C7+D7</f>
         <v>0.43</v>
       </c>
-      <c r="F7" s="13" t="n">
+      <c r="F7" s="12" t="n">
         <f aca="false">$B$4*(1-E7)</f>
-        <v>301833.077142857</v>
-      </c>
-      <c r="G7" s="13" t="n">
-        <f aca="false">F7-LandedCost!J4</f>
-        <v>65133.0771428572</v>
-      </c>
-      <c r="H7" s="20" t="n">
+        <v>301738.969491429</v>
+      </c>
+      <c r="G7" s="12" t="n">
+        <f aca="false">F7-LandedCost!K4</f>
+        <v>65112.7694914286</v>
+      </c>
+      <c r="H7" s="22" t="n">
         <f aca="false">IF(F7=0,0,G7/F7)</f>
         <v>0.215791714279313</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="7" t="s">
-        <v>97</v>
-      </c>
-      <c r="B8" s="9" t="n">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="B8" s="8" t="n">
         <v>0.18</v>
       </c>
-      <c r="C8" s="9" t="n">
+      <c r="C8" s="8" t="n">
         <v>0.18</v>
       </c>
-      <c r="D8" s="9" t="n">
+      <c r="D8" s="8" t="n">
         <v>0.05</v>
       </c>
-      <c r="E8" s="20" t="n">
+      <c r="E8" s="22" t="n">
         <f aca="false">B8+C8+D8</f>
         <v>0.41</v>
       </c>
-      <c r="F8" s="13" t="n">
+      <c r="F8" s="12" t="n">
         <f aca="false">$B$4*(1-E8)</f>
-        <v>312423.711428572</v>
-      </c>
-      <c r="G8" s="13" t="n">
-        <f aca="false">F8-LandedCost!J4</f>
-        <v>75723.7114285715</v>
-      </c>
-      <c r="H8" s="20" t="n">
+        <v>312326.301754286</v>
+      </c>
+      <c r="G8" s="12" t="n">
+        <f aca="false">F8-LandedCost!K4</f>
+        <v>75700.1017542858</v>
+      </c>
+      <c r="H8" s="22" t="n">
         <f aca="false">IF(F8=0,0,G8/F8)</f>
         <v>0.242375045998658</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="7" t="s">
-        <v>98</v>
-      </c>
-      <c r="B9" s="9" t="n">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="B9" s="8" t="n">
         <v>0.15</v>
       </c>
-      <c r="C9" s="9" t="n">
+      <c r="C9" s="8" t="n">
         <v>0.05</v>
       </c>
-      <c r="D9" s="9" t="n">
+      <c r="D9" s="8" t="n">
         <v>0.03</v>
       </c>
-      <c r="E9" s="20" t="n">
+      <c r="E9" s="22" t="n">
         <f aca="false">B9+C9+D9</f>
         <v>0.23</v>
       </c>
-      <c r="F9" s="13" t="n">
+      <c r="F9" s="12" t="n">
         <f aca="false">$B$4*(1-E9)</f>
-        <v>407739.42</v>
-      </c>
-      <c r="G9" s="13" t="n">
-        <f aca="false">F9-LandedCost!J4</f>
-        <v>171039.42</v>
-      </c>
-      <c r="H9" s="20" t="n">
+        <v>407612.29212</v>
+      </c>
+      <c r="G9" s="12" t="n">
+        <f aca="false">F9-LandedCost!K4</f>
+        <v>170986.09212</v>
+      </c>
+      <c r="H9" s="22" t="n">
         <f aca="false">IF(F9=0,0,G9/F9)</f>
         <v>0.419482178102868</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7" t="s">
-        <v>99</v>
-      </c>
-      <c r="B10" s="9" t="n">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="B10" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="C10" s="9" t="n">
+      <c r="C10" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="D10" s="9" t="n">
+      <c r="D10" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="E10" s="20" t="n">
+      <c r="E10" s="22" t="n">
         <f aca="false">B10+C10+D10</f>
         <v>0</v>
       </c>
-      <c r="F10" s="13" t="n">
+      <c r="F10" s="12" t="n">
         <f aca="false">$B$4*(1-E10)</f>
-        <v>529531.714285714</v>
-      </c>
-      <c r="G10" s="13" t="n">
-        <f aca="false">F10-LandedCost!J4</f>
-        <v>292831.714285714</v>
-      </c>
-      <c r="H10" s="20" t="n">
+        <v>529366.613142857</v>
+      </c>
+      <c r="G10" s="12" t="n">
+        <f aca="false">F10-LandedCost!K4</f>
+        <v>292740.413142857</v>
+      </c>
+      <c r="H10" s="22" t="n">
         <f aca="false">IF(F10=0,0,G10/F10)</f>
         <v>0.553001277139208</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="s">
-        <v>100</v>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="2" t="s">
+        <v>103</v>
       </c>
     </row>
   </sheetData>
@@ -2362,201 +2435,201 @@
   <dimension ref="A1:I16"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="1" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="13"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="I1" s="21" t="n">
-        <f aca="false">LandedCost!C4</f>
-        <v>12</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="5" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="22" t="s">
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="B4" s="22" t="s">
+      <c r="H1" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="C4" s="22" t="s">
-        <v>60</v>
-      </c>
-      <c r="D4" s="22" t="s">
-        <v>77</v>
-      </c>
-      <c r="E4" s="22" t="s">
-        <v>79</v>
-      </c>
-      <c r="F4" s="22" t="s">
+      <c r="I1" s="23" t="n">
+        <f aca="false">LandedCost!D4</f>
+        <v>11.996</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="4" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="24" t="s">
+        <v>107</v>
+      </c>
+      <c r="B4" s="24" t="s">
+        <v>108</v>
+      </c>
+      <c r="C4" s="24" t="s">
+        <v>63</v>
+      </c>
+      <c r="D4" s="24" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="7" t="s">
-        <v>106</v>
-      </c>
-      <c r="B5" s="23" t="n">
+      <c r="E4" s="24" t="s">
+        <v>82</v>
+      </c>
+      <c r="F4" s="24" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="B5" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="C5" s="13" t="n">
-        <f aca="false">(LandedCost!D4+Controls!$B$8)*(1+B5)+Controls!$B$17/Controls!$B$18</f>
-        <v>236700</v>
-      </c>
-      <c r="D5" s="13" t="n">
+      <c r="C5" s="12" t="n">
+        <f aca="false">(LandedCost!E4+Controls!$B$8)*(1+B5)+Controls!$B$17/Controls!$B$18</f>
+        <v>236626.2</v>
+      </c>
+      <c r="D5" s="12" t="n">
         <f aca="false">(C5*(1+Controls!$B$13)/(1-Controls!$B$14))*(1+Controls!$B$10)</f>
-        <v>529531.714285714</v>
-      </c>
-      <c r="E5" s="15" t="n">
+        <v>529366.613142857</v>
+      </c>
+      <c r="E5" s="16" t="n">
         <f aca="false">D5/Controls!$B$4</f>
-        <v>28.700905923345</v>
-      </c>
-      <c r="F5" s="16" t="n">
-        <f aca="false">D5/LandedCost!D4</f>
-        <v>2.39174216027875</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="7" t="s">
-        <v>107</v>
-      </c>
-      <c r="B6" s="23" t="n">
+        <v>28.6919573519164</v>
+      </c>
+      <c r="F5" s="17" t="n">
+        <f aca="false">D5/LandedCost!E4</f>
+        <v>2.39179371056322</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="B6" s="25" t="n">
         <v>0.15</v>
       </c>
-      <c r="C6" s="13" t="n">
-        <f aca="false">(LandedCost!D4+Controls!$B$8)*(1+B6)+Controls!$B$17/Controls!$B$18</f>
-        <v>271680</v>
-      </c>
-      <c r="D6" s="13" t="n">
+      <c r="C6" s="12" t="n">
+        <f aca="false">(LandedCost!E4+Controls!$B$8)*(1+B6)+Controls!$B$17/Controls!$B$18</f>
+        <v>271595.13</v>
+      </c>
+      <c r="D6" s="12" t="n">
         <f aca="false">(C6*(1+Controls!$B$13)/(1-Controls!$B$14))*(1+Controls!$B$10)</f>
-        <v>607786.971428572</v>
-      </c>
-      <c r="E6" s="15" t="n">
+        <v>607597.105114286</v>
+      </c>
+      <c r="E6" s="16" t="n">
         <f aca="false">D6/Controls!$B$4</f>
-        <v>32.9423832752613</v>
-      </c>
-      <c r="F6" s="16" t="n">
-        <f aca="false">D6/LandedCost!D4</f>
-        <v>2.74519860627178</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="7" t="s">
-        <v>108</v>
-      </c>
-      <c r="B7" s="23" t="n">
+        <v>32.9320924181185</v>
+      </c>
+      <c r="F6" s="17" t="n">
+        <f aca="false">D6/LandedCost!E4</f>
+        <v>2.74525612021661</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="B7" s="25" t="n">
         <v>0.07</v>
       </c>
-      <c r="C7" s="13" t="n">
-        <f aca="false">(LandedCost!D4+Controls!$B$8)*(1+B7)+Controls!$B$17/Controls!$B$18</f>
-        <v>253024</v>
-      </c>
-      <c r="D7" s="13" t="n">
+      <c r="C7" s="12" t="n">
+        <f aca="false">(LandedCost!E4+Controls!$B$8)*(1+B7)+Controls!$B$17/Controls!$B$18</f>
+        <v>252945.034</v>
+      </c>
+      <c r="D7" s="12" t="n">
         <f aca="false">(C7*(1+Controls!$B$13)/(1-Controls!$B$14))*(1+Controls!$B$10)</f>
-        <v>566050.834285714</v>
-      </c>
-      <c r="E7" s="15" t="n">
+        <v>565874.176062857</v>
+      </c>
+      <c r="E7" s="16" t="n">
         <f aca="false">D7/Controls!$B$4</f>
-        <v>30.6802620209059</v>
-      </c>
-      <c r="F7" s="16" t="n">
-        <f aca="false">D7/LandedCost!D4</f>
-        <v>2.55668850174216</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="5" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="24" t="s">
+        <v>30.6706870494774</v>
+      </c>
+      <c r="F7" s="17" t="n">
+        <f aca="false">D7/LandedCost!E4</f>
+        <v>2.55674283506814</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="26" t="s">
         <v>39</v>
       </c>
-      <c r="B11" s="24" t="s">
-        <v>77</v>
-      </c>
-      <c r="C11" s="24" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="17" t="n">
+      <c r="B11" s="26" t="s">
+        <v>80</v>
+      </c>
+      <c r="C11" s="26" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="18" t="n">
         <v>17500</v>
       </c>
-      <c r="B12" s="13" t="n">
-        <f aca="false">((LandedCost!C4*A12+Controls!$B$8)+Controls!$B$17/Controls!$B$18)*(1+Controls!$B$13)/(1-Controls!$B$14)*(1+Controls!$B$10)</f>
-        <v>504028.285714286</v>
-      </c>
-      <c r="C12" s="15" t="n">
+      <c r="B12" s="12" t="n">
+        <f aca="false">((LandedCost!D4*A12+Controls!$B$8)+Controls!$B$17/Controls!$B$18)*(1+Controls!$B$13)/(1-Controls!$B$14)*(1+Controls!$B$10)</f>
+        <v>503871.685714286</v>
+      </c>
+      <c r="C12" s="16" t="n">
         <f aca="false">B12/A12</f>
-        <v>28.8016163265306</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="17" t="n">
+        <v>28.792667755102</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="18" t="n">
         <v>18000</v>
       </c>
-      <c r="B13" s="13" t="n">
-        <f aca="false">((LandedCost!C4*A13+Controls!$B$8)+Controls!$B$17/Controls!$B$18)*(1+Controls!$B$13)/(1-Controls!$B$14)*(1+Controls!$B$10)</f>
-        <v>517451.142857143</v>
-      </c>
-      <c r="C13" s="15" t="n">
+      <c r="B13" s="12" t="n">
+        <f aca="false">((LandedCost!D4*A13+Controls!$B$8)+Controls!$B$17/Controls!$B$18)*(1+Controls!$B$13)/(1-Controls!$B$14)*(1+Controls!$B$10)</f>
+        <v>517290.068571429</v>
+      </c>
+      <c r="C13" s="16" t="n">
         <f aca="false">B13/A13</f>
-        <v>28.7472857142857</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="17" t="n">
+        <v>28.7383371428571</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="18" t="n">
         <v>18450</v>
       </c>
-      <c r="B14" s="13" t="n">
-        <f aca="false">((LandedCost!C4*A14+Controls!$B$8)+Controls!$B$17/Controls!$B$18)*(1+Controls!$B$13)/(1-Controls!$B$14)*(1+Controls!$B$10)</f>
-        <v>529531.714285714</v>
-      </c>
-      <c r="C14" s="15" t="n">
+      <c r="B14" s="12" t="n">
+        <f aca="false">((LandedCost!D4*A14+Controls!$B$8)+Controls!$B$17/Controls!$B$18)*(1+Controls!$B$13)/(1-Controls!$B$14)*(1+Controls!$B$10)</f>
+        <v>529366.613142857</v>
+      </c>
+      <c r="C14" s="16" t="n">
         <f aca="false">B14/A14</f>
-        <v>28.700905923345</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="17" t="n">
+        <v>28.6919573519164</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="18" t="n">
         <v>19000</v>
       </c>
-      <c r="B15" s="13" t="n">
-        <f aca="false">((LandedCost!C4*A15+Controls!$B$8)+Controls!$B$17/Controls!$B$18)*(1+Controls!$B$13)/(1-Controls!$B$14)*(1+Controls!$B$10)</f>
-        <v>544296.857142857</v>
-      </c>
-      <c r="C15" s="15" t="n">
+      <c r="B15" s="12" t="n">
+        <f aca="false">((LandedCost!D4*A15+Controls!$B$8)+Controls!$B$17/Controls!$B$18)*(1+Controls!$B$13)/(1-Controls!$B$14)*(1+Controls!$B$10)</f>
+        <v>544126.834285714</v>
+      </c>
+      <c r="C15" s="16" t="n">
         <f aca="false">B15/A15</f>
-        <v>28.6472030075188</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="17" t="n">
+        <v>28.6382544360902</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="18" t="n">
         <v>19500</v>
       </c>
-      <c r="B16" s="13" t="n">
-        <f aca="false">((LandedCost!C4*A16+Controls!$B$8)+Controls!$B$17/Controls!$B$18)*(1+Controls!$B$13)/(1-Controls!$B$14)*(1+Controls!$B$10)</f>
-        <v>557719.714285714</v>
-      </c>
-      <c r="C16" s="15" t="n">
+      <c r="B16" s="12" t="n">
+        <f aca="false">((LandedCost!D4*A16+Controls!$B$8)+Controls!$B$17/Controls!$B$18)*(1+Controls!$B$13)/(1-Controls!$B$14)*(1+Controls!$B$10)</f>
+        <v>557545.217142857</v>
+      </c>
+      <c r="C16" s="16" t="n">
         <f aca="false">B16/A16</f>
-        <v>28.601010989011</v>
+        <v>28.5920624175824</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Model: add Organika pricing method, channel calibration, pack lever
FOB now follows Organika's pricing method when real COGS is entered
(price = COGS / (1 - 45% CM - 10% trade)), falling back to Canadian
retail x 40% until then. Adds a channel-multiple check (shelf at 3x
and 4x Organika price, per the observed Vietnam channel markup of
200-300%) and a per-SKU pack factor for Vietnam-specific sizes.
Workbook marked INTERNAL. 160 formulas, zero errors; COGS path and
pack factor tested.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CHL2VrJ5edbBW6zFNsXfxt
</commit_message>
<xml_diff>
--- a/vietnam-margin-model.xlsx
+++ b/vietnam-margin-model.xlsx
@@ -146,7 +146,55 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Rule of thumb (LOW): brand wholesale ~50% of retail; export FOB at or below domestic wholesale. Replace with Organika export price list.</t>
+          <t xml:space="preserve">Fallback only, used when a SKU has no COGS entered. Rule of thumb (LOW).</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B22" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Organika internal pricing method for this account, Oct 2026: start at 45% CM.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B23" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Organika internal pricing method, Oct 2026: 10% trade spend. Price = COGS / (1 - CM - trade).</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B26" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Vietnam channel markup recalled as 200-300% in Oct 2026 (retail = 3x to 4x Organika price). On-file average not yet checked (LOW-MEDIUM).</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B27" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">See above.</t>
         </r>
       </text>
     </comment>
@@ -232,6 +280,150 @@
         </r>
       </text>
     </comment>
+    <comment ref="L4" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Enter real COGS (CAD/unit). When filled, FOB = COGS/(1-CM-trade) per Organika pricing method; when blank, falls back to retail x ratio.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="L5" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Enter real COGS (CAD/unit). When filled, FOB = COGS/(1-CM-trade) per Organika pricing method; when blank, falls back to retail x ratio.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="L6" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Enter real COGS (CAD/unit). When filled, FOB = COGS/(1-CM-trade) per Organika pricing method; when blank, falls back to retail x ratio.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="L7" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Enter real COGS (CAD/unit). When filled, FOB = COGS/(1-CM-trade) per Organika pricing method; when blank, falls back to retail x ratio.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="L8" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Enter real COGS (CAD/unit). When filled, FOB = COGS/(1-CM-trade) per Organika pricing method; when blank, falls back to retail x ratio.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="L9" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Enter real COGS (CAD/unit). When filled, FOB = COGS/(1-CM-trade) per Organika pricing method; when blank, falls back to retail x ratio.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="M4" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Scale for a Vietnam specific pack, e.g. 0.5 for a half size pack. New pack = new registration, label and MOQ.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="M5" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Scale for a Vietnam specific pack, e.g. 0.5 for a half size pack. New pack = new registration, label and MOQ.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="M6" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Scale for a Vietnam specific pack, e.g. 0.5 for a half size pack. New pack = new registration, label and MOQ.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="M7" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Scale for a Vietnam specific pack, e.g. 0.5 for a half size pack. New pack = new registration, label and MOQ.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="M8" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Scale for a Vietnam specific pack, e.g. 0.5 for a half size pack. New pack = new registration, label and MOQ.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="M9" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Scale for a Vietnam specific pack, e.g. 0.5 for a half size pack. New pack = new registration, label and MOQ.</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
@@ -319,7 +511,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="129">
   <si>
     <t xml:space="preserve">Organika — Vietnam Landed Cost &amp; Margin Model</t>
   </si>
@@ -429,7 +621,19 @@
     <t xml:space="preserve">FOB costs</t>
   </si>
   <si>
-    <t xml:space="preserve">ESTIMATED: Canadian retail (real 2026 shelf prices) x export FOB ratio (40%, rule of thumb) on Controls. Probiotic and vitamin C retail are placeholders. Replace with the Organika export price list.</t>
+    <t xml:space="preserve">Enter real COGS per SKU on LandedCost (column L): FOB then follows Organika pricing method, COGS/(1-45%-10%). Until then FOB falls back to Canadian retail x 40% (LOW).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Channel check</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Observed Vietnam channel markup 200-300% (retail 3x to 4x Organika price), recalled Oct 2026, not yet checked against the on-file average (LOW-MEDIUM).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confidentiality</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INTERNAL. Contains Organika pricing policy. Do not share outside Organika, including with distributors.</t>
   </si>
   <si>
     <t xml:space="preserve">Controls — set once, drives every tab</t>
@@ -480,7 +684,25 @@
     <t xml:space="preserve">Export pricing</t>
   </si>
   <si>
-    <t xml:space="preserve">Export FOB as % of Canadian retail</t>
+    <t xml:space="preserve">Export FOB as % of Canadian retail (fallback)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Target contribution margin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trade spend</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Channel calibration</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Channel multiple, low (shelf / Organika price)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Channel multiple, high</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INTERNAL: contains Organika pricing policy. Do not share this workbook outside Organika.</t>
   </si>
   <si>
     <t xml:space="preserve">Landed cost per unit (CIF + duty), by SKU</t>
@@ -519,6 +741,12 @@
     <t xml:space="preserve">Landed+Reg (VND)</t>
   </si>
   <si>
+    <t xml:space="preserve">COGS (CAD) — enter real</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pack factor (1 = Canadian pack)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Enhanced Collagen (250g)</t>
   </si>
   <si>
@@ -549,12 +777,15 @@
     <t xml:space="preserve">Vitamin C / dailies</t>
   </si>
   <si>
-    <t xml:space="preserve">Canadian retail: real 2026 shelf prices (hover for source); yellow = placeholder. FOB = retail x export ratio on Controls (rule of thumb, replace with Organika export price list).</t>
+    <t xml:space="preserve">FOB: COGS/(1-CM-trade) when real COGS is entered (column L), else Canadian retail x fallback ratio. Canadian retail = real 2026 shelf prices (hover). Yellow = placeholder or required input.</t>
   </si>
   <si>
     <t xml:space="preserve">SKU economics — shelf price vs the real Vietnamese shelf</t>
   </si>
   <si>
+    <t xml:space="preserve">Two lenses: the modeled margin stack (columns B to K) and the observed Vietnam channel multiple of 3x to 4x Organika price (columns M to O). Trust the stricter one until real COGS and on-file markups are in.</t>
+  </si>
+  <si>
     <t xml:space="preserve">To distributor (VND)</t>
   </si>
   <si>
@@ -579,10 +810,19 @@
     <t xml:space="preserve">Comparable band high (VND)</t>
   </si>
   <si>
-    <t xml:space="preserve">Position</t>
+    <t xml:space="preserve">Position (model stack)</t>
   </si>
   <si>
     <t xml:space="preserve">Max FOB to hit band midpoint (CAD)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shelf at channel 3x (VND)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shelf at channel 4x (VND)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Position at 3x to 4x</t>
   </si>
   <si>
     <t xml:space="preserve">Channel economics — what the brand nets per unit</t>
@@ -664,16 +904,17 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="7">
+  <numFmts count="8">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
-    <numFmt numFmtId="167" formatCode="0.00"/>
-    <numFmt numFmtId="168" formatCode="\$#,##0.0"/>
-    <numFmt numFmtId="169" formatCode="&quot;C$&quot;#,##0.0"/>
-    <numFmt numFmtId="170" formatCode="0.00\x"/>
+    <numFmt numFmtId="167" formatCode="0.0\x"/>
+    <numFmt numFmtId="168" formatCode="0.00"/>
+    <numFmt numFmtId="169" formatCode="\$#,##0.0"/>
+    <numFmt numFmtId="170" formatCode="&quot;C$&quot;#,##0.0"/>
+    <numFmt numFmtId="171" formatCode="0.00\x"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -737,6 +978,14 @@
     <font>
       <sz val="10"/>
       <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="10"/>
+      <color rgb="FFB3402F"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -831,7 +1080,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="29">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -868,15 +1117,23 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -884,15 +1141,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -904,6 +1157,10 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="171" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="165" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -912,11 +1169,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -924,11 +1181,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -936,7 +1193,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1003,7 +1260,7 @@
       <rgbColor rgb="FF339966"/>
       <rgbColor rgb="FF003300"/>
       <rgbColor rgb="FF333300"/>
-      <rgbColor rgb="FF993300"/>
+      <rgbColor rgb="FFB3402F"/>
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF333399"/>
       <rgbColor rgb="FF1F4D3A"/>
@@ -1192,7 +1449,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B24"/>
+  <dimension ref="A1:B26"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20"/>
@@ -1365,6 +1622,22 @@
       </c>
       <c r="B24" s="3" t="s">
         <v>36</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>40</v>
       </c>
     </row>
   </sheetData>
@@ -1383,7 +1656,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
@@ -1392,142 +1665,196 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="B4" s="7" t="n">
         <v>18450</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="B5" s="7" t="n">
         <v>26200</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="B8" s="7" t="n">
         <v>11800</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="B9" s="8" t="n">
         <v>0</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="B10" s="8" t="n">
         <v>0.08</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="B13" s="8" t="n">
         <v>0.45</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="B14" s="8" t="n">
         <v>0.3</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="B17" s="7" t="n">
         <v>70000000</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="B18" s="7" t="n">
         <v>20000</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="B21" s="8" t="n">
         <v>0.4</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>40</v>
+        <v>44</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="B22" s="8" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="B23" s="8" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="4" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="B26" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="B27" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="10" t="s">
+        <v>63</v>
       </c>
     </row>
   </sheetData>
@@ -1547,7 +1874,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:M11"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
@@ -1558,309 +1885,340 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="0" width="13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="12" style="0" width="14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>54</v>
+        <v>64</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="B3" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="C3" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="D3" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="E3" s="9" t="s">
-        <v>59</v>
-      </c>
-      <c r="F3" s="9" t="s">
-        <v>60</v>
-      </c>
-      <c r="G3" s="9" t="s">
-        <v>61</v>
-      </c>
-      <c r="H3" s="9" t="s">
-        <v>62</v>
-      </c>
-      <c r="I3" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="J3" s="9" t="s">
-        <v>64</v>
-      </c>
-      <c r="K3" s="9" t="s">
+      <c r="A3" s="11" t="s">
         <v>65</v>
+      </c>
+      <c r="B3" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="D3" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="E3" s="11" t="s">
+        <v>69</v>
+      </c>
+      <c r="F3" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="G3" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="H3" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="I3" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="J3" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="K3" s="11" t="s">
+        <v>75</v>
+      </c>
+      <c r="L3" s="11" t="s">
+        <v>76</v>
+      </c>
+      <c r="M3" s="11" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>66</v>
+        <v>78</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="C4" s="10" t="n">
+        <v>79</v>
+      </c>
+      <c r="C4" s="12" t="n">
         <v>29.99</v>
       </c>
-      <c r="D4" s="11" t="n">
-        <f aca="false">C4*Controls!$B$21</f>
+      <c r="D4" s="13" t="n">
+        <f aca="false">IF(N(L4)&gt;0,L4/(1-Controls!$B$22-Controls!$B$23),C4*Controls!$B$21)*M4</f>
         <v>11.996</v>
       </c>
-      <c r="E4" s="12" t="n">
+      <c r="E4" s="14" t="n">
         <f aca="false">D4*Controls!$B$4</f>
         <v>221326.2</v>
       </c>
-      <c r="F4" s="13" t="n">
+      <c r="F4" s="15" t="n">
         <f aca="false">Controls!$B$8</f>
         <v>11800</v>
       </c>
-      <c r="G4" s="12" t="n">
+      <c r="G4" s="14" t="n">
         <f aca="false">E4+F4</f>
         <v>233126.2</v>
       </c>
-      <c r="H4" s="12" t="n">
+      <c r="H4" s="14" t="n">
         <f aca="false">G4*Controls!$B$9</f>
         <v>0</v>
       </c>
-      <c r="I4" s="12" t="n">
+      <c r="I4" s="14" t="n">
         <f aca="false">G4+H4</f>
         <v>233126.2</v>
       </c>
-      <c r="J4" s="13" t="n">
+      <c r="J4" s="15" t="n">
         <f aca="false">Controls!$B$17/Controls!$B$18</f>
         <v>3500</v>
       </c>
-      <c r="K4" s="12" t="n">
+      <c r="K4" s="14" t="n">
         <f aca="false">I4+J4</f>
         <v>236626.2</v>
       </c>
+      <c r="L4" s="16"/>
+      <c r="M4" s="12" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="C5" s="10" t="n">
+        <v>81</v>
+      </c>
+      <c r="C5" s="12" t="n">
         <v>27.99</v>
       </c>
-      <c r="D5" s="11" t="n">
-        <f aca="false">C5*Controls!$B$21</f>
+      <c r="D5" s="13" t="n">
+        <f aca="false">IF(N(L5)&gt;0,L5/(1-Controls!$B$22-Controls!$B$23),C5*Controls!$B$21)*M5</f>
         <v>11.196</v>
       </c>
-      <c r="E5" s="12" t="n">
+      <c r="E5" s="14" t="n">
         <f aca="false">D5*Controls!$B$4</f>
         <v>206566.2</v>
       </c>
-      <c r="F5" s="13" t="n">
+      <c r="F5" s="15" t="n">
         <f aca="false">Controls!$B$8</f>
         <v>11800</v>
       </c>
-      <c r="G5" s="12" t="n">
+      <c r="G5" s="14" t="n">
         <f aca="false">E5+F5</f>
         <v>218366.2</v>
       </c>
-      <c r="H5" s="12" t="n">
+      <c r="H5" s="14" t="n">
         <f aca="false">G5*Controls!$B$9</f>
         <v>0</v>
       </c>
-      <c r="I5" s="12" t="n">
+      <c r="I5" s="14" t="n">
         <f aca="false">G5+H5</f>
         <v>218366.2</v>
       </c>
-      <c r="J5" s="13" t="n">
+      <c r="J5" s="15" t="n">
         <f aca="false">Controls!$B$17/Controls!$B$18</f>
         <v>3500</v>
       </c>
-      <c r="K5" s="12" t="n">
+      <c r="K5" s="14" t="n">
         <f aca="false">I5+J5</f>
         <v>221866.2</v>
       </c>
+      <c r="L5" s="16"/>
+      <c r="M5" s="12" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>70</v>
+        <v>82</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="C6" s="10" t="n">
+        <v>81</v>
+      </c>
+      <c r="C6" s="12" t="n">
         <v>43.49</v>
       </c>
-      <c r="D6" s="11" t="n">
-        <f aca="false">C6*Controls!$B$21</f>
+      <c r="D6" s="13" t="n">
+        <f aca="false">IF(N(L6)&gt;0,L6/(1-Controls!$B$22-Controls!$B$23),C6*Controls!$B$21)*M6</f>
         <v>17.396</v>
       </c>
-      <c r="E6" s="12" t="n">
+      <c r="E6" s="14" t="n">
         <f aca="false">D6*Controls!$B$4</f>
         <v>320956.2</v>
       </c>
-      <c r="F6" s="13" t="n">
+      <c r="F6" s="15" t="n">
         <f aca="false">Controls!$B$8</f>
         <v>11800</v>
       </c>
-      <c r="G6" s="12" t="n">
+      <c r="G6" s="14" t="n">
         <f aca="false">E6+F6</f>
         <v>332756.2</v>
       </c>
-      <c r="H6" s="12" t="n">
+      <c r="H6" s="14" t="n">
         <f aca="false">G6*Controls!$B$9</f>
         <v>0</v>
       </c>
-      <c r="I6" s="12" t="n">
+      <c r="I6" s="14" t="n">
         <f aca="false">G6+H6</f>
         <v>332756.2</v>
       </c>
-      <c r="J6" s="13" t="n">
+      <c r="J6" s="15" t="n">
         <f aca="false">Controls!$B$17/Controls!$B$18</f>
         <v>3500</v>
       </c>
-      <c r="K6" s="12" t="n">
+      <c r="K6" s="14" t="n">
         <f aca="false">I6+J6</f>
         <v>336256.2</v>
       </c>
+      <c r="L6" s="16"/>
+      <c r="M6" s="12" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>71</v>
+        <v>83</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="C7" s="10" t="n">
+        <v>84</v>
+      </c>
+      <c r="C7" s="12" t="n">
         <v>25.99</v>
       </c>
-      <c r="D7" s="11" t="n">
-        <f aca="false">C7*Controls!$B$21</f>
+      <c r="D7" s="13" t="n">
+        <f aca="false">IF(N(L7)&gt;0,L7/(1-Controls!$B$22-Controls!$B$23),C7*Controls!$B$21)*M7</f>
         <v>10.396</v>
       </c>
-      <c r="E7" s="12" t="n">
+      <c r="E7" s="14" t="n">
         <f aca="false">D7*Controls!$B$4</f>
         <v>191806.2</v>
       </c>
-      <c r="F7" s="13" t="n">
+      <c r="F7" s="15" t="n">
         <f aca="false">Controls!$B$8</f>
         <v>11800</v>
       </c>
-      <c r="G7" s="12" t="n">
+      <c r="G7" s="14" t="n">
         <f aca="false">E7+F7</f>
         <v>203606.2</v>
       </c>
-      <c r="H7" s="12" t="n">
+      <c r="H7" s="14" t="n">
         <f aca="false">G7*Controls!$B$9</f>
         <v>0</v>
       </c>
-      <c r="I7" s="12" t="n">
+      <c r="I7" s="14" t="n">
         <f aca="false">G7+H7</f>
         <v>203606.2</v>
       </c>
-      <c r="J7" s="13" t="n">
+      <c r="J7" s="15" t="n">
         <f aca="false">Controls!$B$17/Controls!$B$18</f>
         <v>3500</v>
       </c>
-      <c r="K7" s="12" t="n">
+      <c r="K7" s="14" t="n">
         <f aca="false">I7+J7</f>
         <v>207106.2</v>
       </c>
+      <c r="L7" s="16"/>
+      <c r="M7" s="12" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>73</v>
+        <v>85</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="C8" s="14" t="n">
+        <v>86</v>
+      </c>
+      <c r="C8" s="16" t="n">
         <v>35</v>
       </c>
-      <c r="D8" s="11" t="n">
-        <f aca="false">C8*Controls!$B$21</f>
+      <c r="D8" s="13" t="n">
+        <f aca="false">IF(N(L8)&gt;0,L8/(1-Controls!$B$22-Controls!$B$23),C8*Controls!$B$21)*M8</f>
         <v>14</v>
       </c>
-      <c r="E8" s="12" t="n">
+      <c r="E8" s="14" t="n">
         <f aca="false">D8*Controls!$B$4</f>
         <v>258300</v>
       </c>
-      <c r="F8" s="13" t="n">
+      <c r="F8" s="15" t="n">
         <f aca="false">Controls!$B$8</f>
         <v>11800</v>
       </c>
-      <c r="G8" s="12" t="n">
+      <c r="G8" s="14" t="n">
         <f aca="false">E8+F8</f>
         <v>270100</v>
       </c>
-      <c r="H8" s="12" t="n">
+      <c r="H8" s="14" t="n">
         <f aca="false">G8*Controls!$B$9</f>
         <v>0</v>
       </c>
-      <c r="I8" s="12" t="n">
+      <c r="I8" s="14" t="n">
         <f aca="false">G8+H8</f>
         <v>270100</v>
       </c>
-      <c r="J8" s="13" t="n">
+      <c r="J8" s="15" t="n">
         <f aca="false">Controls!$B$17/Controls!$B$18</f>
         <v>3500</v>
       </c>
-      <c r="K8" s="12" t="n">
+      <c r="K8" s="14" t="n">
         <f aca="false">I8+J8</f>
         <v>273600</v>
       </c>
+      <c r="L8" s="16"/>
+      <c r="M8" s="12" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>75</v>
+        <v>87</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="C9" s="14" t="n">
+        <v>84</v>
+      </c>
+      <c r="C9" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="D9" s="11" t="n">
-        <f aca="false">C9*Controls!$B$21</f>
+      <c r="D9" s="13" t="n">
+        <f aca="false">IF(N(L9)&gt;0,L9/(1-Controls!$B$22-Controls!$B$23),C9*Controls!$B$21)*M9</f>
         <v>6</v>
       </c>
-      <c r="E9" s="12" t="n">
+      <c r="E9" s="14" t="n">
         <f aca="false">D9*Controls!$B$4</f>
         <v>110700</v>
       </c>
-      <c r="F9" s="13" t="n">
+      <c r="F9" s="15" t="n">
         <f aca="false">Controls!$B$8</f>
         <v>11800</v>
       </c>
-      <c r="G9" s="12" t="n">
+      <c r="G9" s="14" t="n">
         <f aca="false">E9+F9</f>
         <v>122500</v>
       </c>
-      <c r="H9" s="12" t="n">
+      <c r="H9" s="14" t="n">
         <f aca="false">G9*Controls!$B$9</f>
         <v>0</v>
       </c>
-      <c r="I9" s="12" t="n">
+      <c r="I9" s="14" t="n">
         <f aca="false">G9+H9</f>
         <v>122500</v>
       </c>
-      <c r="J9" s="13" t="n">
+      <c r="J9" s="15" t="n">
         <f aca="false">Controls!$B$17/Controls!$B$18</f>
         <v>3500</v>
       </c>
-      <c r="K9" s="12" t="n">
+      <c r="K9" s="14" t="n">
         <f aca="false">I9+J9</f>
         <v>126000</v>
       </c>
+      <c r="L9" s="16"/>
+      <c r="M9" s="12" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>76</v>
+        <v>88</v>
       </c>
     </row>
   </sheetData>
@@ -1880,7 +2238,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:O9"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
@@ -1890,333 +2248,421 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="6" style="0" width="11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="28"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="13" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="26"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>77</v>
+        <v>89</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="B3" s="9" t="s">
+      <c r="A3" s="11" t="s">
         <v>65</v>
       </c>
-      <c r="C3" s="9" t="s">
-        <v>78</v>
-      </c>
-      <c r="D3" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="E3" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="F3" s="9" t="s">
-        <v>81</v>
-      </c>
-      <c r="G3" s="9" t="s">
-        <v>82</v>
-      </c>
-      <c r="H3" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="I3" s="9" t="s">
-        <v>84</v>
-      </c>
-      <c r="J3" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="K3" s="9" t="s">
-        <v>86</v>
-      </c>
-      <c r="L3" s="9" t="s">
-        <v>87</v>
+      <c r="B3" s="11" t="s">
+        <v>75</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="D3" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="E3" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="F3" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="G3" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="H3" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="I3" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="J3" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="K3" s="11" t="s">
+        <v>99</v>
+      </c>
+      <c r="L3" s="11" t="s">
+        <v>100</v>
+      </c>
+      <c r="M3" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="N3" s="11" t="s">
+        <v>102</v>
+      </c>
+      <c r="O3" s="11" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="B4" s="13" t="n">
+        <v>78</v>
+      </c>
+      <c r="B4" s="15" t="n">
         <f aca="false">LandedCost!K4</f>
         <v>236626.2</v>
       </c>
-      <c r="C4" s="12" t="n">
+      <c r="C4" s="14" t="n">
         <f aca="false">B4*(1+Controls!$B$13)</f>
         <v>343107.99</v>
       </c>
-      <c r="D4" s="12" t="n">
+      <c r="D4" s="14" t="n">
         <f aca="false">C4/(1-Controls!$B$14)</f>
         <v>490154.271428571</v>
       </c>
-      <c r="E4" s="12" t="n">
+      <c r="E4" s="14" t="n">
         <f aca="false">D4*(1+Controls!$B$10)</f>
         <v>529366.613142857</v>
       </c>
-      <c r="F4" s="15" t="n">
+      <c r="F4" s="17" t="n">
         <f aca="false">E4/Controls!$B$5</f>
         <v>20.2048325627045</v>
       </c>
-      <c r="G4" s="16" t="n">
+      <c r="G4" s="18" t="n">
         <f aca="false">E4/Controls!$B$4</f>
         <v>28.6919573519164</v>
       </c>
-      <c r="H4" s="17" t="n">
+      <c r="H4" s="19" t="n">
         <f aca="false">E4/LandedCost!E4</f>
         <v>2.39179371056322</v>
       </c>
-      <c r="I4" s="18" t="n">
+      <c r="I4" s="20" t="n">
         <v>650000</v>
       </c>
-      <c r="J4" s="18" t="n">
+      <c r="J4" s="20" t="n">
         <v>850000</v>
       </c>
-      <c r="K4" s="19" t="str">
+      <c r="K4" s="21" t="str">
         <f aca="false">IF(E4&lt;I4,"Below band — room to price up",IF(E4&gt;J4,"Above band — promo-room risk","Within band"))</f>
         <v>Below band — room to price up</v>
       </c>
-      <c r="L4" s="20" t="n">
+      <c r="L4" s="22" t="n">
         <f aca="false">(((I4+J4)/2/((1+Controls!$B$13)/(1-Controls!$B$14)*(1+Controls!$B$10))-Controls!$B$17/Controls!$B$18)/(1+Controls!$B$9)-Controls!$B$8)/Controls!$B$4</f>
         <v>17.3414114984062</v>
       </c>
+      <c r="M4" s="14" t="n">
+        <f aca="false">LandedCost!E4*Controls!$B$26</f>
+        <v>663978.6</v>
+      </c>
+      <c r="N4" s="14" t="n">
+        <f aca="false">LandedCost!E4*Controls!$B$27</f>
+        <v>885304.8</v>
+      </c>
+      <c r="O4" s="21" t="str">
+        <f aca="false">IF(N4&lt;I4,"Below band",IF(M4&gt;J4,"Above band at both multiples",IF(AND(M4&gt;=I4,N4&lt;=J4),"In band at both","Straddles band")))</f>
+        <v>Straddles band</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="B5" s="13" t="n">
+        <v>80</v>
+      </c>
+      <c r="B5" s="15" t="n">
         <f aca="false">LandedCost!K5</f>
         <v>221866.2</v>
       </c>
-      <c r="C5" s="12" t="n">
+      <c r="C5" s="14" t="n">
         <f aca="false">B5*(1+Controls!$B$13)</f>
         <v>321705.99</v>
       </c>
-      <c r="D5" s="12" t="n">
+      <c r="D5" s="14" t="n">
         <f aca="false">C5/(1-Controls!$B$14)</f>
         <v>459579.985714286</v>
       </c>
-      <c r="E5" s="12" t="n">
+      <c r="E5" s="14" t="n">
         <f aca="false">D5*(1+Controls!$B$10)</f>
         <v>496346.384571429</v>
       </c>
-      <c r="F5" s="15" t="n">
+      <c r="F5" s="17" t="n">
         <f aca="false">E5/Controls!$B$5</f>
         <v>18.9445184950927</v>
       </c>
-      <c r="G5" s="16" t="n">
+      <c r="G5" s="18" t="n">
         <f aca="false">E5/Controls!$B$4</f>
         <v>26.9022430662021</v>
       </c>
-      <c r="H5" s="17" t="n">
+      <c r="H5" s="19" t="n">
         <f aca="false">E5/LandedCost!E5</f>
         <v>2.40284414667757</v>
       </c>
-      <c r="I5" s="18" t="n">
+      <c r="I5" s="20" t="n">
         <v>220000</v>
       </c>
-      <c r="J5" s="18" t="n">
+      <c r="J5" s="20" t="n">
         <v>500000</v>
       </c>
-      <c r="K5" s="19" t="str">
+      <c r="K5" s="21" t="str">
         <f aca="false">IF(E5&lt;I5,"Below band — room to price up",IF(E5&gt;J5,"Above band — promo-room risk","Within band"))</f>
         <v>Within band</v>
       </c>
-      <c r="L5" s="20" t="n">
+      <c r="L5" s="22" t="n">
         <f aca="false">(((I5+J5)/2/((1+Controls!$B$13)/(1-Controls!$B$14)*(1+Controls!$B$10))-Controls!$B$17/Controls!$B$18)/(1+Controls!$B$9)-Controls!$B$8)/Controls!$B$4</f>
         <v>7.89265800703984</v>
       </c>
+      <c r="M5" s="14" t="n">
+        <f aca="false">LandedCost!E5*Controls!$B$26</f>
+        <v>619698.6</v>
+      </c>
+      <c r="N5" s="14" t="n">
+        <f aca="false">LandedCost!E5*Controls!$B$27</f>
+        <v>826264.8</v>
+      </c>
+      <c r="O5" s="21" t="str">
+        <f aca="false">IF(N5&lt;I5,"Below band",IF(M5&gt;J5,"Above band at both multiples",IF(AND(M5&gt;=I5,N5&lt;=J5),"In band at both","Straddles band")))</f>
+        <v>Above band at both multiples</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="B6" s="13" t="n">
+        <v>82</v>
+      </c>
+      <c r="B6" s="15" t="n">
         <f aca="false">LandedCost!K6</f>
         <v>336256.2</v>
       </c>
-      <c r="C6" s="12" t="n">
+      <c r="C6" s="14" t="n">
         <f aca="false">B6*(1+Controls!$B$13)</f>
         <v>487571.49</v>
       </c>
-      <c r="D6" s="12" t="n">
+      <c r="D6" s="14" t="n">
         <f aca="false">C6/(1-Controls!$B$14)</f>
         <v>696530.7</v>
       </c>
-      <c r="E6" s="12" t="n">
+      <c r="E6" s="14" t="n">
         <f aca="false">D6*(1+Controls!$B$10)</f>
         <v>752253.156</v>
       </c>
-      <c r="F6" s="15" t="n">
+      <c r="F6" s="17" t="n">
         <f aca="false">E6/Controls!$B$5</f>
         <v>28.711952519084</v>
       </c>
-      <c r="G6" s="16" t="n">
+      <c r="G6" s="18" t="n">
         <f aca="false">E6/Controls!$B$4</f>
         <v>40.7725287804878</v>
       </c>
-      <c r="H6" s="17" t="n">
+      <c r="H6" s="19" t="n">
         <f aca="false">E6/LandedCost!E6</f>
         <v>2.34378758223085</v>
       </c>
-      <c r="I6" s="18" t="n">
+      <c r="I6" s="20" t="n">
         <v>350000</v>
       </c>
-      <c r="J6" s="18" t="n">
+      <c r="J6" s="20" t="n">
         <v>600000</v>
       </c>
-      <c r="K6" s="19" t="str">
+      <c r="K6" s="21" t="str">
         <f aca="false">IF(E6&lt;I6,"Below band — room to price up",IF(E6&gt;J6,"Above band — promo-room risk","Within band"))</f>
         <v>Above band — promo-room risk</v>
       </c>
-      <c r="L6" s="20" t="n">
+      <c r="L6" s="22" t="n">
         <f aca="false">(((I6+J6)/2/((1+Controls!$B$13)/(1-Controls!$B$14)*(1+Controls!$B$10))-Controls!$B$17/Controls!$B$18)/(1+Controls!$B$9)-Controls!$B$8)/Controls!$B$4</f>
         <v>10.6788289083402</v>
       </c>
+      <c r="M6" s="14" t="n">
+        <f aca="false">LandedCost!E6*Controls!$B$26</f>
+        <v>962868.6</v>
+      </c>
+      <c r="N6" s="14" t="n">
+        <f aca="false">LandedCost!E6*Controls!$B$27</f>
+        <v>1283824.8</v>
+      </c>
+      <c r="O6" s="21" t="str">
+        <f aca="false">IF(N6&lt;I6,"Below band",IF(M6&gt;J6,"Above band at both multiples",IF(AND(M6&gt;=I6,N6&lt;=J6),"In band at both","Straddles band")))</f>
+        <v>Above band at both multiples</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="B7" s="13" t="n">
+        <v>83</v>
+      </c>
+      <c r="B7" s="15" t="n">
         <f aca="false">LandedCost!K7</f>
         <v>207106.2</v>
       </c>
-      <c r="C7" s="12" t="n">
+      <c r="C7" s="14" t="n">
         <f aca="false">B7*(1+Controls!$B$13)</f>
         <v>300303.99</v>
       </c>
-      <c r="D7" s="12" t="n">
+      <c r="D7" s="14" t="n">
         <f aca="false">C7/(1-Controls!$B$14)</f>
         <v>429005.7</v>
       </c>
-      <c r="E7" s="12" t="n">
+      <c r="E7" s="14" t="n">
         <f aca="false">D7*(1+Controls!$B$10)</f>
         <v>463326.156</v>
       </c>
-      <c r="F7" s="15" t="n">
+      <c r="F7" s="17" t="n">
         <f aca="false">E7/Controls!$B$5</f>
         <v>17.6842044274809</v>
       </c>
-      <c r="G7" s="16" t="n">
+      <c r="G7" s="18" t="n">
         <f aca="false">E7/Controls!$B$4</f>
         <v>25.1125287804878</v>
       </c>
-      <c r="H7" s="17" t="n">
+      <c r="H7" s="19" t="n">
         <f aca="false">E7/LandedCost!E7</f>
         <v>2.41559530400999</v>
       </c>
-      <c r="I7" s="18" t="n">
+      <c r="I7" s="20" t="n">
         <v>250000</v>
       </c>
-      <c r="J7" s="18" t="n">
+      <c r="J7" s="20" t="n">
         <v>400000</v>
       </c>
-      <c r="K7" s="19" t="str">
+      <c r="K7" s="21" t="str">
         <f aca="false">IF(E7&lt;I7,"Below band — room to price up",IF(E7&gt;J7,"Above band — promo-room risk","Within band"))</f>
         <v>Above band — promo-room risk</v>
       </c>
-      <c r="L7" s="20" t="n">
+      <c r="L7" s="22" t="n">
         <f aca="false">(((I7+J7)/2/((1+Controls!$B$13)/(1-Controls!$B$14)*(1+Controls!$B$10))-Controls!$B$17/Controls!$B$18)/(1+Controls!$B$9)-Controls!$B$8)/Controls!$B$4</f>
         <v>7.04469295012235</v>
       </c>
+      <c r="M7" s="14" t="n">
+        <f aca="false">LandedCost!E7*Controls!$B$26</f>
+        <v>575418.6</v>
+      </c>
+      <c r="N7" s="14" t="n">
+        <f aca="false">LandedCost!E7*Controls!$B$27</f>
+        <v>767224.8</v>
+      </c>
+      <c r="O7" s="21" t="str">
+        <f aca="false">IF(N7&lt;I7,"Below band",IF(M7&gt;J7,"Above band at both multiples",IF(AND(M7&gt;=I7,N7&lt;=J7),"In band at both","Straddles band")))</f>
+        <v>Above band at both multiples</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>73</v>
-      </c>
-      <c r="B8" s="13" t="n">
+        <v>85</v>
+      </c>
+      <c r="B8" s="15" t="n">
         <f aca="false">LandedCost!K8</f>
         <v>273600</v>
       </c>
-      <c r="C8" s="12" t="n">
+      <c r="C8" s="14" t="n">
         <f aca="false">B8*(1+Controls!$B$13)</f>
         <v>396720</v>
       </c>
-      <c r="D8" s="12" t="n">
+      <c r="D8" s="14" t="n">
         <f aca="false">C8/(1-Controls!$B$14)</f>
         <v>566742.857142857</v>
       </c>
-      <c r="E8" s="12" t="n">
+      <c r="E8" s="14" t="n">
         <f aca="false">D8*(1+Controls!$B$10)</f>
         <v>612082.285714286</v>
       </c>
-      <c r="F8" s="15" t="n">
+      <c r="F8" s="17" t="n">
         <f aca="false">E8/Controls!$B$5</f>
         <v>23.361919302072</v>
       </c>
-      <c r="G8" s="16" t="n">
+      <c r="G8" s="18" t="n">
         <f aca="false">E8/Controls!$B$4</f>
         <v>33.1751916376307</v>
       </c>
-      <c r="H8" s="17" t="n">
+      <c r="H8" s="19" t="n">
         <f aca="false">E8/LandedCost!E8</f>
         <v>2.36965654554505</v>
       </c>
-      <c r="I8" s="18" t="n">
+      <c r="I8" s="20" t="n">
         <v>350000</v>
       </c>
-      <c r="J8" s="18" t="n">
+      <c r="J8" s="20" t="n">
         <v>550000</v>
       </c>
-      <c r="K8" s="19" t="str">
+      <c r="K8" s="21" t="str">
         <f aca="false">IF(E8&lt;I8,"Below band — room to price up",IF(E8&gt;J8,"Above band — promo-room risk","Within band"))</f>
         <v>Above band — promo-room risk</v>
       </c>
-      <c r="L8" s="20" t="n">
+      <c r="L8" s="22" t="n">
         <f aca="false">(((I8+J8)/2/((1+Controls!$B$13)/(1-Controls!$B$14)*(1+Controls!$B$10))-Controls!$B$17/Controls!$B$18)/(1+Controls!$B$9)-Controls!$B$8)/Controls!$B$4</f>
         <v>10.0731395819705</v>
       </c>
+      <c r="M8" s="14" t="n">
+        <f aca="false">LandedCost!E8*Controls!$B$26</f>
+        <v>774900</v>
+      </c>
+      <c r="N8" s="14" t="n">
+        <f aca="false">LandedCost!E8*Controls!$B$27</f>
+        <v>1033200</v>
+      </c>
+      <c r="O8" s="21" t="str">
+        <f aca="false">IF(N8&lt;I8,"Below band",IF(M8&gt;J8,"Above band at both multiples",IF(AND(M8&gt;=I8,N8&lt;=J8),"In band at both","Straddles band")))</f>
+        <v>Above band at both multiples</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="B9" s="13" t="n">
+        <v>87</v>
+      </c>
+      <c r="B9" s="15" t="n">
         <f aca="false">LandedCost!K9</f>
         <v>126000</v>
       </c>
-      <c r="C9" s="12" t="n">
+      <c r="C9" s="14" t="n">
         <f aca="false">B9*(1+Controls!$B$13)</f>
         <v>182700</v>
       </c>
-      <c r="D9" s="12" t="n">
+      <c r="D9" s="14" t="n">
         <f aca="false">C9/(1-Controls!$B$14)</f>
         <v>261000</v>
       </c>
-      <c r="E9" s="12" t="n">
+      <c r="E9" s="14" t="n">
         <f aca="false">D9*(1+Controls!$B$10)</f>
         <v>281880</v>
       </c>
-      <c r="F9" s="15" t="n">
+      <c r="F9" s="17" t="n">
         <f aca="false">E9/Controls!$B$5</f>
         <v>10.7587786259542</v>
       </c>
-      <c r="G9" s="16" t="n">
+      <c r="G9" s="18" t="n">
         <f aca="false">E9/Controls!$B$4</f>
         <v>15.2780487804878</v>
       </c>
-      <c r="H9" s="17" t="n">
+      <c r="H9" s="19" t="n">
         <f aca="false">E9/LandedCost!E9</f>
         <v>2.54634146341463</v>
       </c>
-      <c r="I9" s="18" t="n">
+      <c r="I9" s="20" t="n">
         <v>60000</v>
       </c>
-      <c r="J9" s="18" t="n">
+      <c r="J9" s="20" t="n">
         <v>150000</v>
       </c>
-      <c r="K9" s="19" t="str">
+      <c r="K9" s="21" t="str">
         <f aca="false">IF(E9&lt;I9,"Below band — room to price up",IF(E9&gt;J9,"Above band — promo-room risk","Within band"))</f>
         <v>Above band — promo-room risk</v>
       </c>
-      <c r="L9" s="20" t="n">
+      <c r="L9" s="22" t="n">
         <f aca="false">(((I9+J9)/2/((1+Controls!$B$13)/(1-Controls!$B$14)*(1+Controls!$B$10))-Controls!$B$17/Controls!$B$18)/(1+Controls!$B$9)-Controls!$B$8)/Controls!$B$4</f>
         <v>1.71462687806955</v>
+      </c>
+      <c r="M9" s="14" t="n">
+        <f aca="false">LandedCost!E9*Controls!$B$26</f>
+        <v>332100</v>
+      </c>
+      <c r="N9" s="14" t="n">
+        <f aca="false">LandedCost!E9*Controls!$B$27</f>
+        <v>442800</v>
+      </c>
+      <c r="O9" s="21" t="str">
+        <f aca="false">IF(N9&lt;I9,"Below band",IF(M9&gt;J9,"Above band at both multiples",IF(AND(M9&gt;=I9,N9&lt;=J9),"In band at both","Straddles band")))</f>
+        <v>Above band at both multiples</v>
       </c>
     </row>
   </sheetData>
@@ -2248,52 +2694,52 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>88</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>89</v>
+        <v>105</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="B4" s="21" t="n">
+        <v>106</v>
+      </c>
+      <c r="B4" s="23" t="n">
         <f aca="false">SKU_Economics!E4</f>
         <v>529366.613142857</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="9" t="s">
-        <v>91</v>
-      </c>
-      <c r="B6" s="9" t="s">
-        <v>92</v>
-      </c>
-      <c r="C6" s="9" t="s">
-        <v>93</v>
-      </c>
-      <c r="D6" s="9" t="s">
-        <v>94</v>
-      </c>
-      <c r="E6" s="9" t="s">
-        <v>95</v>
-      </c>
-      <c r="F6" s="9" t="s">
-        <v>96</v>
-      </c>
-      <c r="G6" s="9" t="s">
-        <v>97</v>
-      </c>
-      <c r="H6" s="9" t="s">
-        <v>98</v>
+      <c r="A6" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>108</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="D6" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="E6" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="F6" s="11" t="s">
+        <v>112</v>
+      </c>
+      <c r="G6" s="11" t="s">
+        <v>113</v>
+      </c>
+      <c r="H6" s="11" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="B7" s="8" t="n">
         <v>0.21</v>
@@ -2304,26 +2750,26 @@
       <c r="D7" s="8" t="n">
         <v>0.07</v>
       </c>
-      <c r="E7" s="22" t="n">
+      <c r="E7" s="24" t="n">
         <f aca="false">B7+C7+D7</f>
         <v>0.43</v>
       </c>
-      <c r="F7" s="12" t="n">
+      <c r="F7" s="14" t="n">
         <f aca="false">$B$4*(1-E7)</f>
         <v>301738.969491429</v>
       </c>
-      <c r="G7" s="12" t="n">
+      <c r="G7" s="14" t="n">
         <f aca="false">F7-LandedCost!K4</f>
         <v>65112.7694914286</v>
       </c>
-      <c r="H7" s="22" t="n">
+      <c r="H7" s="24" t="n">
         <f aca="false">IF(F7=0,0,G7/F7)</f>
         <v>0.215791714279313</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>100</v>
+        <v>116</v>
       </c>
       <c r="B8" s="8" t="n">
         <v>0.18</v>
@@ -2334,26 +2780,26 @@
       <c r="D8" s="8" t="n">
         <v>0.05</v>
       </c>
-      <c r="E8" s="22" t="n">
+      <c r="E8" s="24" t="n">
         <f aca="false">B8+C8+D8</f>
         <v>0.41</v>
       </c>
-      <c r="F8" s="12" t="n">
+      <c r="F8" s="14" t="n">
         <f aca="false">$B$4*(1-E8)</f>
         <v>312326.301754286</v>
       </c>
-      <c r="G8" s="12" t="n">
+      <c r="G8" s="14" t="n">
         <f aca="false">F8-LandedCost!K4</f>
         <v>75700.1017542858</v>
       </c>
-      <c r="H8" s="22" t="n">
+      <c r="H8" s="24" t="n">
         <f aca="false">IF(F8=0,0,G8/F8)</f>
         <v>0.242375045998658</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>101</v>
+        <v>117</v>
       </c>
       <c r="B9" s="8" t="n">
         <v>0.15</v>
@@ -2364,26 +2810,26 @@
       <c r="D9" s="8" t="n">
         <v>0.03</v>
       </c>
-      <c r="E9" s="22" t="n">
+      <c r="E9" s="24" t="n">
         <f aca="false">B9+C9+D9</f>
         <v>0.23</v>
       </c>
-      <c r="F9" s="12" t="n">
+      <c r="F9" s="14" t="n">
         <f aca="false">$B$4*(1-E9)</f>
         <v>407612.29212</v>
       </c>
-      <c r="G9" s="12" t="n">
+      <c r="G9" s="14" t="n">
         <f aca="false">F9-LandedCost!K4</f>
         <v>170986.09212</v>
       </c>
-      <c r="H9" s="22" t="n">
+      <c r="H9" s="24" t="n">
         <f aca="false">IF(F9=0,0,G9/F9)</f>
         <v>0.419482178102868</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>102</v>
+        <v>118</v>
       </c>
       <c r="B10" s="8" t="n">
         <v>0</v>
@@ -2394,26 +2840,26 @@
       <c r="D10" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="E10" s="22" t="n">
+      <c r="E10" s="24" t="n">
         <f aca="false">B10+C10+D10</f>
         <v>0</v>
       </c>
-      <c r="F10" s="12" t="n">
+      <c r="F10" s="14" t="n">
         <f aca="false">$B$4*(1-E10)</f>
         <v>529366.613142857</v>
       </c>
-      <c r="G10" s="12" t="n">
+      <c r="G10" s="14" t="n">
         <f aca="false">F10-LandedCost!K4</f>
         <v>292740.413142857</v>
       </c>
-      <c r="H10" s="22" t="n">
+      <c r="H10" s="24" t="n">
         <f aca="false">IF(F10=0,0,G10/F10)</f>
         <v>0.553001277139208</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>103</v>
+        <v>119</v>
       </c>
     </row>
   </sheetData>
@@ -2444,190 +2890,190 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>104</v>
+        <v>120</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="I1" s="23" t="n">
+        <v>121</v>
+      </c>
+      <c r="I1" s="25" t="n">
         <f aca="false">LandedCost!D4</f>
         <v>11.996</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>106</v>
+        <v>122</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="24" t="s">
-        <v>107</v>
-      </c>
-      <c r="B4" s="24" t="s">
-        <v>108</v>
-      </c>
-      <c r="C4" s="24" t="s">
-        <v>63</v>
-      </c>
-      <c r="D4" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="E4" s="24" t="s">
-        <v>82</v>
-      </c>
-      <c r="F4" s="24" t="s">
-        <v>83</v>
+      <c r="A4" s="26" t="s">
+        <v>123</v>
+      </c>
+      <c r="B4" s="26" t="s">
+        <v>124</v>
+      </c>
+      <c r="C4" s="26" t="s">
+        <v>73</v>
+      </c>
+      <c r="D4" s="26" t="s">
+        <v>93</v>
+      </c>
+      <c r="E4" s="26" t="s">
+        <v>95</v>
+      </c>
+      <c r="F4" s="26" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>109</v>
-      </c>
-      <c r="B5" s="25" t="n">
+        <v>125</v>
+      </c>
+      <c r="B5" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="C5" s="12" t="n">
+      <c r="C5" s="14" t="n">
         <f aca="false">(LandedCost!E4+Controls!$B$8)*(1+B5)+Controls!$B$17/Controls!$B$18</f>
         <v>236626.2</v>
       </c>
-      <c r="D5" s="12" t="n">
+      <c r="D5" s="14" t="n">
         <f aca="false">(C5*(1+Controls!$B$13)/(1-Controls!$B$14))*(1+Controls!$B$10)</f>
         <v>529366.613142857</v>
       </c>
-      <c r="E5" s="16" t="n">
+      <c r="E5" s="18" t="n">
         <f aca="false">D5/Controls!$B$4</f>
         <v>28.6919573519164</v>
       </c>
-      <c r="F5" s="17" t="n">
+      <c r="F5" s="19" t="n">
         <f aca="false">D5/LandedCost!E4</f>
         <v>2.39179371056322</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>110</v>
-      </c>
-      <c r="B6" s="25" t="n">
+        <v>126</v>
+      </c>
+      <c r="B6" s="27" t="n">
         <v>0.15</v>
       </c>
-      <c r="C6" s="12" t="n">
+      <c r="C6" s="14" t="n">
         <f aca="false">(LandedCost!E4+Controls!$B$8)*(1+B6)+Controls!$B$17/Controls!$B$18</f>
         <v>271595.13</v>
       </c>
-      <c r="D6" s="12" t="n">
+      <c r="D6" s="14" t="n">
         <f aca="false">(C6*(1+Controls!$B$13)/(1-Controls!$B$14))*(1+Controls!$B$10)</f>
         <v>607597.105114286</v>
       </c>
-      <c r="E6" s="16" t="n">
+      <c r="E6" s="18" t="n">
         <f aca="false">D6/Controls!$B$4</f>
         <v>32.9320924181185</v>
       </c>
-      <c r="F6" s="17" t="n">
+      <c r="F6" s="19" t="n">
         <f aca="false">D6/LandedCost!E4</f>
         <v>2.74525612021661</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>111</v>
-      </c>
-      <c r="B7" s="25" t="n">
+        <v>127</v>
+      </c>
+      <c r="B7" s="27" t="n">
         <v>0.07</v>
       </c>
-      <c r="C7" s="12" t="n">
+      <c r="C7" s="14" t="n">
         <f aca="false">(LandedCost!E4+Controls!$B$8)*(1+B7)+Controls!$B$17/Controls!$B$18</f>
         <v>252945.034</v>
       </c>
-      <c r="D7" s="12" t="n">
+      <c r="D7" s="14" t="n">
         <f aca="false">(C7*(1+Controls!$B$13)/(1-Controls!$B$14))*(1+Controls!$B$10)</f>
         <v>565874.176062857</v>
       </c>
-      <c r="E7" s="16" t="n">
+      <c r="E7" s="18" t="n">
         <f aca="false">D7/Controls!$B$4</f>
         <v>30.6706870494774</v>
       </c>
-      <c r="F7" s="17" t="n">
+      <c r="F7" s="19" t="n">
         <f aca="false">D7/LandedCost!E4</f>
         <v>2.55674283506814</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>112</v>
+        <v>128</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="26" t="s">
-        <v>39</v>
-      </c>
-      <c r="B11" s="26" t="s">
-        <v>80</v>
-      </c>
-      <c r="C11" s="26" t="s">
-        <v>82</v>
+      <c r="A11" s="28" t="s">
+        <v>43</v>
+      </c>
+      <c r="B11" s="28" t="s">
+        <v>93</v>
+      </c>
+      <c r="C11" s="28" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="18" t="n">
+      <c r="A12" s="20" t="n">
         <v>17500</v>
       </c>
-      <c r="B12" s="12" t="n">
+      <c r="B12" s="14" t="n">
         <f aca="false">((LandedCost!D4*A12+Controls!$B$8)+Controls!$B$17/Controls!$B$18)*(1+Controls!$B$13)/(1-Controls!$B$14)*(1+Controls!$B$10)</f>
         <v>503871.685714286</v>
       </c>
-      <c r="C12" s="16" t="n">
+      <c r="C12" s="18" t="n">
         <f aca="false">B12/A12</f>
         <v>28.792667755102</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="18" t="n">
+      <c r="A13" s="20" t="n">
         <v>18000</v>
       </c>
-      <c r="B13" s="12" t="n">
+      <c r="B13" s="14" t="n">
         <f aca="false">((LandedCost!D4*A13+Controls!$B$8)+Controls!$B$17/Controls!$B$18)*(1+Controls!$B$13)/(1-Controls!$B$14)*(1+Controls!$B$10)</f>
         <v>517290.068571429</v>
       </c>
-      <c r="C13" s="16" t="n">
+      <c r="C13" s="18" t="n">
         <f aca="false">B13/A13</f>
         <v>28.7383371428571</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="18" t="n">
+      <c r="A14" s="20" t="n">
         <v>18450</v>
       </c>
-      <c r="B14" s="12" t="n">
+      <c r="B14" s="14" t="n">
         <f aca="false">((LandedCost!D4*A14+Controls!$B$8)+Controls!$B$17/Controls!$B$18)*(1+Controls!$B$13)/(1-Controls!$B$14)*(1+Controls!$B$10)</f>
         <v>529366.613142857</v>
       </c>
-      <c r="C14" s="16" t="n">
+      <c r="C14" s="18" t="n">
         <f aca="false">B14/A14</f>
         <v>28.6919573519164</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="18" t="n">
+      <c r="A15" s="20" t="n">
         <v>19000</v>
       </c>
-      <c r="B15" s="12" t="n">
+      <c r="B15" s="14" t="n">
         <f aca="false">((LandedCost!D4*A15+Controls!$B$8)+Controls!$B$17/Controls!$B$18)*(1+Controls!$B$13)/(1-Controls!$B$14)*(1+Controls!$B$10)</f>
         <v>544126.834285714</v>
       </c>
-      <c r="C15" s="16" t="n">
+      <c r="C15" s="18" t="n">
         <f aca="false">B15/A15</f>
         <v>28.6382544360902</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="18" t="n">
+      <c r="A16" s="20" t="n">
         <v>19500</v>
       </c>
-      <c r="B16" s="12" t="n">
+      <c r="B16" s="14" t="n">
         <f aca="false">((LandedCost!D4*A16+Controls!$B$8)+Controls!$B$17/Controls!$B$18)*(1+Controls!$B$13)/(1-Controls!$B$14)*(1+Controls!$B$10)</f>
         <v>557545.217142857</v>
       </c>
-      <c r="C16" s="16" t="n">
+      <c r="C16" s="18" t="n">
         <f aca="false">B16/A16</f>
         <v>28.5920624175824</v>
       </c>

</xml_diff>

<commit_message>
Remove internal pricing and channel details from public files
Margin targets and channel multiples are now blank, guarded inputs in the
model; primer, app, playbook, README and exec summary use neutral wording.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CHL2VrJ5edbBW6zFNsXfxt
</commit_message>
<xml_diff>
--- a/vietnam-margin-model.xlsx
+++ b/vietnam-margin-model.xlsx
@@ -158,7 +158,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Organika internal pricing method for this account, Oct 2026: start at 45% CM.</t>
+          <t xml:space="preserve">Enter your own target. Blank = FOB uses the retail fallback.</t>
         </r>
       </text>
     </comment>
@@ -170,7 +170,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Organika internal pricing method, Oct 2026: 10% trade spend. Price = COGS / (1 - CM - trade).</t>
+          <t xml:space="preserve">Enter your own trade spend. Price = COGS / (1 - margin - trade).</t>
         </r>
       </text>
     </comment>
@@ -182,7 +182,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Vietnam channel markup recalled as 200-300% in Oct 2026 (retail = 3x to 4x Organika price). On-file average not yet checked (LOW-MEDIUM).</t>
+          <t xml:space="preserve">Optional. Enter your account's actual multiple; blank hides this lens.</t>
         </r>
       </text>
     </comment>
@@ -194,7 +194,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">See above.</t>
+          <t xml:space="preserve">Optional. See above.</t>
         </r>
       </text>
     </comment>
@@ -288,7 +288,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Enter real COGS (CAD/unit). When filled, FOB = COGS/(1-CM-trade) per Organika pricing method; when blank, falls back to retail x ratio.</t>
+          <t xml:space="preserve">Enter real COGS (CAD/unit). When filled with margin and trade targets on Controls, FOB = COGS/(1-margin-trade); otherwise, falls back to retail x ratio.</t>
         </r>
       </text>
     </comment>
@@ -300,7 +300,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Enter real COGS (CAD/unit). When filled, FOB = COGS/(1-CM-trade) per Organika pricing method; when blank, falls back to retail x ratio.</t>
+          <t xml:space="preserve">Enter real COGS (CAD/unit). When filled with margin and trade targets on Controls, FOB = COGS/(1-margin-trade); otherwise, falls back to retail x ratio.</t>
         </r>
       </text>
     </comment>
@@ -312,7 +312,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Enter real COGS (CAD/unit). When filled, FOB = COGS/(1-CM-trade) per Organika pricing method; when blank, falls back to retail x ratio.</t>
+          <t xml:space="preserve">Enter real COGS (CAD/unit). When filled with margin and trade targets on Controls, FOB = COGS/(1-margin-trade); otherwise, falls back to retail x ratio.</t>
         </r>
       </text>
     </comment>
@@ -324,7 +324,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Enter real COGS (CAD/unit). When filled, FOB = COGS/(1-CM-trade) per Organika pricing method; when blank, falls back to retail x ratio.</t>
+          <t xml:space="preserve">Enter real COGS (CAD/unit). When filled with margin and trade targets on Controls, FOB = COGS/(1-margin-trade); otherwise, falls back to retail x ratio.</t>
         </r>
       </text>
     </comment>
@@ -336,7 +336,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Enter real COGS (CAD/unit). When filled, FOB = COGS/(1-CM-trade) per Organika pricing method; when blank, falls back to retail x ratio.</t>
+          <t xml:space="preserve">Enter real COGS (CAD/unit). When filled with margin and trade targets on Controls, FOB = COGS/(1-margin-trade); otherwise, falls back to retail x ratio.</t>
         </r>
       </text>
     </comment>
@@ -348,7 +348,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Enter real COGS (CAD/unit). When filled, FOB = COGS/(1-CM-trade) per Organika pricing method; when blank, falls back to retail x ratio.</t>
+          <t xml:space="preserve">Enter real COGS (CAD/unit). When filled with margin and trade targets on Controls, FOB = COGS/(1-margin-trade); otherwise, falls back to retail x ratio.</t>
         </r>
       </text>
     </comment>
@@ -621,19 +621,19 @@
     <t xml:space="preserve">FOB costs</t>
   </si>
   <si>
-    <t xml:space="preserve">Enter real COGS per SKU on LandedCost (column L): FOB then follows Organika pricing method, COGS/(1-45%-10%). Until then FOB falls back to Canadian retail x 40% (LOW).</t>
+    <t xml:space="preserve">Enter real COGS per SKU on LandedCost (column L) and your margin and trade targets on Controls (B22, B23): FOB then = COGS/(1-margin-trade). Until all are entered, FOB falls back to Canadian retail x 40% (LOW).</t>
   </si>
   <si>
     <t xml:space="preserve">Channel check</t>
   </si>
   <si>
-    <t xml:space="preserve">Observed Vietnam channel markup 200-300% (retail 3x to 4x Organika price), recalled Oct 2026, not yet checked against the on-file average (LOW-MEDIUM).</t>
+    <t xml:space="preserve">Optional: enter your account's actual channel multiple (shelf / brand price) on Controls B26 and B27 to add a second lens on SKU_Economics. Blank by default.</t>
   </si>
   <si>
     <t xml:space="preserve">Confidentiality</t>
   </si>
   <si>
-    <t xml:space="preserve">INTERNAL. Contains Organika pricing policy. Do not share outside Organika, including with distributors.</t>
+    <t xml:space="preserve">Template with public inputs only. Once you enter real COGS, margin targets or channel multiples, treat your copy as internal and never share it with a distributor.</t>
   </si>
   <si>
     <t xml:space="preserve">Controls — set once, drives every tab</t>
@@ -696,13 +696,13 @@
     <t xml:space="preserve">Channel calibration</t>
   </si>
   <si>
-    <t xml:space="preserve">Channel multiple, low (shelf / Organika price)</t>
+    <t xml:space="preserve">Channel multiple, low (shelf / brand price)</t>
   </si>
   <si>
     <t xml:space="preserve">Channel multiple, high</t>
   </si>
   <si>
-    <t xml:space="preserve">INTERNAL: contains Organika pricing policy. Do not share this workbook outside Organika.</t>
+    <t xml:space="preserve">Once real COGS, margins or multiples are entered, treat your copy as internal. Never share it with a distributor.</t>
   </si>
   <si>
     <t xml:space="preserve">Landed cost per unit (CIF + duty), by SKU</t>
@@ -777,13 +777,13 @@
     <t xml:space="preserve">Vitamin C / dailies</t>
   </si>
   <si>
-    <t xml:space="preserve">FOB: COGS/(1-CM-trade) when real COGS is entered (column L), else Canadian retail x fallback ratio. Canadian retail = real 2026 shelf prices (hover). Yellow = placeholder or required input.</t>
+    <t xml:space="preserve">FOB: COGS/(1-margin-trade) when real COGS (column L) and margin targets (Controls) are entered, else Canadian retail x fallback ratio. Canadian retail = real 2026 shelf prices (hover). Yellow = placeholder or required input.</t>
   </si>
   <si>
     <t xml:space="preserve">SKU economics — shelf price vs the real Vietnamese shelf</t>
   </si>
   <si>
-    <t xml:space="preserve">Two lenses: the modeled margin stack (columns B to K) and the observed Vietnam channel multiple of 3x to 4x Organika price (columns M to O). Trust the stricter one until real COGS and on-file markups are in.</t>
+    <t xml:space="preserve">Two lenses: the modeled margin stack (columns B to K) and an optional channel multiple you enter on Controls B26 and B27 (columns M to O). Trust the stricter one once real COGS and markups are in.</t>
   </si>
   <si>
     <t xml:space="preserve">To distributor (VND)</t>
@@ -816,13 +816,13 @@
     <t xml:space="preserve">Max FOB to hit band midpoint (CAD)</t>
   </si>
   <si>
-    <t xml:space="preserve">Shelf at channel 3x (VND)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Shelf at channel 4x (VND)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Position at 3x to 4x</t>
+    <t xml:space="preserve">Shelf at channel multiple low (VND)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shelf at channel multiple high (VND)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Position at channel multiples</t>
   </si>
   <si>
     <t xml:space="preserve">Channel economics — what the brand nets per unit</t>
@@ -1807,9 +1807,7 @@
       <c r="A22" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="B22" s="8" t="n">
-        <v>0.45</v>
-      </c>
+      <c r="B22" s="8"/>
       <c r="D22" s="2" t="s">
         <v>44</v>
       </c>
@@ -1818,9 +1816,7 @@
       <c r="A23" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="B23" s="8" t="n">
-        <v>0.1</v>
-      </c>
+      <c r="B23" s="8"/>
       <c r="D23" s="2" t="s">
         <v>44</v>
       </c>
@@ -1834,9 +1830,7 @@
       <c r="A26" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="B26" s="9" t="n">
-        <v>3</v>
-      </c>
+      <c r="B26" s="9"/>
       <c r="D26" s="2" t="s">
         <v>44</v>
       </c>
@@ -1845,9 +1839,7 @@
       <c r="A27" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="B27" s="9" t="n">
-        <v>4</v>
-      </c>
+      <c r="B27" s="9"/>
       <c r="D27" s="2" t="s">
         <v>44</v>
       </c>
@@ -1945,7 +1937,7 @@
         <v>29.99</v>
       </c>
       <c r="D4" s="13" t="n">
-        <f aca="false">IF(N(L4)&gt;0,L4/(1-Controls!$B$22-Controls!$B$23),C4*Controls!$B$21)*M4</f>
+        <f aca="false">IF(AND(N(L4)&gt;0,N(Controls!$B$22)+N(Controls!$B$23)&gt;0,N(Controls!$B$22)+N(Controls!$B$23)&lt;1),L4/(1-Controls!$B$22-Controls!$B$23),C4*Controls!$B$21)*M4</f>
         <v>11.996</v>
       </c>
       <c r="E4" s="14" t="n">
@@ -1992,7 +1984,7 @@
         <v>27.99</v>
       </c>
       <c r="D5" s="13" t="n">
-        <f aca="false">IF(N(L5)&gt;0,L5/(1-Controls!$B$22-Controls!$B$23),C5*Controls!$B$21)*M5</f>
+        <f aca="false">IF(AND(N(L5)&gt;0,N(Controls!$B$22)+N(Controls!$B$23)&gt;0,N(Controls!$B$22)+N(Controls!$B$23)&lt;1),L5/(1-Controls!$B$22-Controls!$B$23),C5*Controls!$B$21)*M5</f>
         <v>11.196</v>
       </c>
       <c r="E5" s="14" t="n">
@@ -2039,7 +2031,7 @@
         <v>43.49</v>
       </c>
       <c r="D6" s="13" t="n">
-        <f aca="false">IF(N(L6)&gt;0,L6/(1-Controls!$B$22-Controls!$B$23),C6*Controls!$B$21)*M6</f>
+        <f aca="false">IF(AND(N(L6)&gt;0,N(Controls!$B$22)+N(Controls!$B$23)&gt;0,N(Controls!$B$22)+N(Controls!$B$23)&lt;1),L6/(1-Controls!$B$22-Controls!$B$23),C6*Controls!$B$21)*M6</f>
         <v>17.396</v>
       </c>
       <c r="E6" s="14" t="n">
@@ -2086,7 +2078,7 @@
         <v>25.99</v>
       </c>
       <c r="D7" s="13" t="n">
-        <f aca="false">IF(N(L7)&gt;0,L7/(1-Controls!$B$22-Controls!$B$23),C7*Controls!$B$21)*M7</f>
+        <f aca="false">IF(AND(N(L7)&gt;0,N(Controls!$B$22)+N(Controls!$B$23)&gt;0,N(Controls!$B$22)+N(Controls!$B$23)&lt;1),L7/(1-Controls!$B$22-Controls!$B$23),C7*Controls!$B$21)*M7</f>
         <v>10.396</v>
       </c>
       <c r="E7" s="14" t="n">
@@ -2133,7 +2125,7 @@
         <v>35</v>
       </c>
       <c r="D8" s="13" t="n">
-        <f aca="false">IF(N(L8)&gt;0,L8/(1-Controls!$B$22-Controls!$B$23),C8*Controls!$B$21)*M8</f>
+        <f aca="false">IF(AND(N(L8)&gt;0,N(Controls!$B$22)+N(Controls!$B$23)&gt;0,N(Controls!$B$22)+N(Controls!$B$23)&lt;1),L8/(1-Controls!$B$22-Controls!$B$23),C8*Controls!$B$21)*M8</f>
         <v>14</v>
       </c>
       <c r="E8" s="14" t="n">
@@ -2180,7 +2172,7 @@
         <v>15</v>
       </c>
       <c r="D9" s="13" t="n">
-        <f aca="false">IF(N(L9)&gt;0,L9/(1-Controls!$B$22-Controls!$B$23),C9*Controls!$B$21)*M9</f>
+        <f aca="false">IF(AND(N(L9)&gt;0,N(Controls!$B$22)+N(Controls!$B$23)&gt;0,N(Controls!$B$22)+N(Controls!$B$23)&lt;1),L9/(1-Controls!$B$22-Controls!$B$23),C9*Controls!$B$21)*M9</f>
         <v>6</v>
       </c>
       <c r="E9" s="14" t="n">
@@ -2357,17 +2349,17 @@
         <f aca="false">(((I4+J4)/2/((1+Controls!$B$13)/(1-Controls!$B$14)*(1+Controls!$B$10))-Controls!$B$17/Controls!$B$18)/(1+Controls!$B$9)-Controls!$B$8)/Controls!$B$4</f>
         <v>17.3414114984062</v>
       </c>
-      <c r="M4" s="14" t="n">
-        <f aca="false">LandedCost!E4*Controls!$B$26</f>
-        <v>663978.6</v>
-      </c>
-      <c r="N4" s="14" t="n">
-        <f aca="false">LandedCost!E4*Controls!$B$27</f>
-        <v>885304.8</v>
+      <c r="M4" s="14" t="str">
+        <f aca="false">IF(N(Controls!$B$26)&gt;0,LandedCost!E4*Controls!$B$26,"")</f>
+        <v/>
+      </c>
+      <c r="N4" s="14" t="str">
+        <f aca="false">IF(N(Controls!$B$27)&gt;0,LandedCost!E4*Controls!$B$27,"")</f>
+        <v/>
       </c>
       <c r="O4" s="21" t="str">
-        <f aca="false">IF(N4&lt;I4,"Below band",IF(M4&gt;J4,"Above band at both multiples",IF(AND(M4&gt;=I4,N4&lt;=J4),"In band at both","Straddles band")))</f>
-        <v>Straddles band</v>
+        <f aca="false">IF(OR(M4="",N4=""),"Enter channel multiples",IF(N4&lt;I4,"Below band",IF(M4&gt;J4,"Above band at both multiples",IF(AND(M4&gt;=I4,N4&lt;=J4),"In band at both","Straddles band"))))</f>
+        <v>Enter channel multiples</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2416,17 +2408,17 @@
         <f aca="false">(((I5+J5)/2/((1+Controls!$B$13)/(1-Controls!$B$14)*(1+Controls!$B$10))-Controls!$B$17/Controls!$B$18)/(1+Controls!$B$9)-Controls!$B$8)/Controls!$B$4</f>
         <v>7.89265800703984</v>
       </c>
-      <c r="M5" s="14" t="n">
-        <f aca="false">LandedCost!E5*Controls!$B$26</f>
-        <v>619698.6</v>
-      </c>
-      <c r="N5" s="14" t="n">
-        <f aca="false">LandedCost!E5*Controls!$B$27</f>
-        <v>826264.8</v>
+      <c r="M5" s="14" t="str">
+        <f aca="false">IF(N(Controls!$B$26)&gt;0,LandedCost!E5*Controls!$B$26,"")</f>
+        <v/>
+      </c>
+      <c r="N5" s="14" t="str">
+        <f aca="false">IF(N(Controls!$B$27)&gt;0,LandedCost!E5*Controls!$B$27,"")</f>
+        <v/>
       </c>
       <c r="O5" s="21" t="str">
-        <f aca="false">IF(N5&lt;I5,"Below band",IF(M5&gt;J5,"Above band at both multiples",IF(AND(M5&gt;=I5,N5&lt;=J5),"In band at both","Straddles band")))</f>
-        <v>Above band at both multiples</v>
+        <f aca="false">IF(OR(M5="",N5=""),"Enter channel multiples",IF(N5&lt;I5,"Below band",IF(M5&gt;J5,"Above band at both multiples",IF(AND(M5&gt;=I5,N5&lt;=J5),"In band at both","Straddles band"))))</f>
+        <v>Enter channel multiples</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2475,17 +2467,17 @@
         <f aca="false">(((I6+J6)/2/((1+Controls!$B$13)/(1-Controls!$B$14)*(1+Controls!$B$10))-Controls!$B$17/Controls!$B$18)/(1+Controls!$B$9)-Controls!$B$8)/Controls!$B$4</f>
         <v>10.6788289083402</v>
       </c>
-      <c r="M6" s="14" t="n">
-        <f aca="false">LandedCost!E6*Controls!$B$26</f>
-        <v>962868.6</v>
-      </c>
-      <c r="N6" s="14" t="n">
-        <f aca="false">LandedCost!E6*Controls!$B$27</f>
-        <v>1283824.8</v>
+      <c r="M6" s="14" t="str">
+        <f aca="false">IF(N(Controls!$B$26)&gt;0,LandedCost!E6*Controls!$B$26,"")</f>
+        <v/>
+      </c>
+      <c r="N6" s="14" t="str">
+        <f aca="false">IF(N(Controls!$B$27)&gt;0,LandedCost!E6*Controls!$B$27,"")</f>
+        <v/>
       </c>
       <c r="O6" s="21" t="str">
-        <f aca="false">IF(N6&lt;I6,"Below band",IF(M6&gt;J6,"Above band at both multiples",IF(AND(M6&gt;=I6,N6&lt;=J6),"In band at both","Straddles band")))</f>
-        <v>Above band at both multiples</v>
+        <f aca="false">IF(OR(M6="",N6=""),"Enter channel multiples",IF(N6&lt;I6,"Below band",IF(M6&gt;J6,"Above band at both multiples",IF(AND(M6&gt;=I6,N6&lt;=J6),"In band at both","Straddles band"))))</f>
+        <v>Enter channel multiples</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2534,17 +2526,17 @@
         <f aca="false">(((I7+J7)/2/((1+Controls!$B$13)/(1-Controls!$B$14)*(1+Controls!$B$10))-Controls!$B$17/Controls!$B$18)/(1+Controls!$B$9)-Controls!$B$8)/Controls!$B$4</f>
         <v>7.04469295012235</v>
       </c>
-      <c r="M7" s="14" t="n">
-        <f aca="false">LandedCost!E7*Controls!$B$26</f>
-        <v>575418.6</v>
-      </c>
-      <c r="N7" s="14" t="n">
-        <f aca="false">LandedCost!E7*Controls!$B$27</f>
-        <v>767224.8</v>
+      <c r="M7" s="14" t="str">
+        <f aca="false">IF(N(Controls!$B$26)&gt;0,LandedCost!E7*Controls!$B$26,"")</f>
+        <v/>
+      </c>
+      <c r="N7" s="14" t="str">
+        <f aca="false">IF(N(Controls!$B$27)&gt;0,LandedCost!E7*Controls!$B$27,"")</f>
+        <v/>
       </c>
       <c r="O7" s="21" t="str">
-        <f aca="false">IF(N7&lt;I7,"Below band",IF(M7&gt;J7,"Above band at both multiples",IF(AND(M7&gt;=I7,N7&lt;=J7),"In band at both","Straddles band")))</f>
-        <v>Above band at both multiples</v>
+        <f aca="false">IF(OR(M7="",N7=""),"Enter channel multiples",IF(N7&lt;I7,"Below band",IF(M7&gt;J7,"Above band at both multiples",IF(AND(M7&gt;=I7,N7&lt;=J7),"In band at both","Straddles band"))))</f>
+        <v>Enter channel multiples</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2593,17 +2585,17 @@
         <f aca="false">(((I8+J8)/2/((1+Controls!$B$13)/(1-Controls!$B$14)*(1+Controls!$B$10))-Controls!$B$17/Controls!$B$18)/(1+Controls!$B$9)-Controls!$B$8)/Controls!$B$4</f>
         <v>10.0731395819705</v>
       </c>
-      <c r="M8" s="14" t="n">
-        <f aca="false">LandedCost!E8*Controls!$B$26</f>
-        <v>774900</v>
-      </c>
-      <c r="N8" s="14" t="n">
-        <f aca="false">LandedCost!E8*Controls!$B$27</f>
-        <v>1033200</v>
+      <c r="M8" s="14" t="str">
+        <f aca="false">IF(N(Controls!$B$26)&gt;0,LandedCost!E8*Controls!$B$26,"")</f>
+        <v/>
+      </c>
+      <c r="N8" s="14" t="str">
+        <f aca="false">IF(N(Controls!$B$27)&gt;0,LandedCost!E8*Controls!$B$27,"")</f>
+        <v/>
       </c>
       <c r="O8" s="21" t="str">
-        <f aca="false">IF(N8&lt;I8,"Below band",IF(M8&gt;J8,"Above band at both multiples",IF(AND(M8&gt;=I8,N8&lt;=J8),"In band at both","Straddles band")))</f>
-        <v>Above band at both multiples</v>
+        <f aca="false">IF(OR(M8="",N8=""),"Enter channel multiples",IF(N8&lt;I8,"Below band",IF(M8&gt;J8,"Above band at both multiples",IF(AND(M8&gt;=I8,N8&lt;=J8),"In band at both","Straddles band"))))</f>
+        <v>Enter channel multiples</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2652,17 +2644,17 @@
         <f aca="false">(((I9+J9)/2/((1+Controls!$B$13)/(1-Controls!$B$14)*(1+Controls!$B$10))-Controls!$B$17/Controls!$B$18)/(1+Controls!$B$9)-Controls!$B$8)/Controls!$B$4</f>
         <v>1.71462687806955</v>
       </c>
-      <c r="M9" s="14" t="n">
-        <f aca="false">LandedCost!E9*Controls!$B$26</f>
-        <v>332100</v>
-      </c>
-      <c r="N9" s="14" t="n">
-        <f aca="false">LandedCost!E9*Controls!$B$27</f>
-        <v>442800</v>
+      <c r="M9" s="14" t="str">
+        <f aca="false">IF(N(Controls!$B$26)&gt;0,LandedCost!E9*Controls!$B$26,"")</f>
+        <v/>
+      </c>
+      <c r="N9" s="14" t="str">
+        <f aca="false">IF(N(Controls!$B$27)&gt;0,LandedCost!E9*Controls!$B$27,"")</f>
+        <v/>
       </c>
       <c r="O9" s="21" t="str">
-        <f aca="false">IF(N9&lt;I9,"Below band",IF(M9&gt;J9,"Above band at both multiples",IF(AND(M9&gt;=I9,N9&lt;=J9),"In band at both","Straddles band")))</f>
-        <v>Above band at both multiples</v>
+        <f aca="false">IF(OR(M9="",N9=""),"Enter channel multiples",IF(N9&lt;I9,"Below band",IF(M9&gt;J9,"Above band at both multiples",IF(AND(M9&gt;=I9,N9&lt;=J9),"In band at both","Straddles band"))))</f>
+        <v>Enter channel multiples</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Loop R1-R2: decision page first; May 2026 platform fee wave; Long Chau Jun 2026
Primer opens with a dated status box and the decision layer; provenance
moves below it. Shopee Mall health fees corrected to the May 2026 wave
(all in take ~25-27%), Lazada and TikTok dates fixed, worked example and
model channel defaults recomputed.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CHL2VrJ5edbBW6zFNsXfxt
</commit_message>
<xml_diff>
--- a/vietnam-margin-model.xlsx
+++ b/vietnam-margin-model.xlsx
@@ -828,7 +828,7 @@
     <t xml:space="preserve">Channel economics — what the brand nets per unit</t>
   </si>
   <si>
-    <t xml:space="preserve">For the hero SKU at its modeled shelf price. Edit take rates (blue) to your real terms.</t>
+    <t xml:space="preserve">For the hero SKU at its modeled shelf price. Platform take rates reflect the May 2026 fee wave (Shopee Mall health 18.0-20.8% fixed + 6% payment; TikTok Shop Mall ~15.5% + 6%; LazMall 6-13% + 6%). Edit to your real terms.</t>
   </si>
   <si>
     <t xml:space="preserve">Shelf price (hero SKU, from SKU_Economics)</t>
@@ -2734,7 +2734,7 @@
         <v>115</v>
       </c>
       <c r="B7" s="8" t="n">
-        <v>0.21</v>
+        <v>0.26</v>
       </c>
       <c r="C7" s="8" t="n">
         <v>0.15</v>
@@ -2744,19 +2744,19 @@
       </c>
       <c r="E7" s="24" t="n">
         <f aca="false">B7+C7+D7</f>
-        <v>0.43</v>
+        <v>0.48</v>
       </c>
       <c r="F7" s="14" t="n">
         <f aca="false">$B$4*(1-E7)</f>
-        <v>301738.969491429</v>
+        <v>275270.638834286</v>
       </c>
       <c r="G7" s="14" t="n">
         <f aca="false">F7-LandedCost!K4</f>
-        <v>65112.7694914286</v>
+        <v>38644.4388342858</v>
       </c>
       <c r="H7" s="24" t="n">
         <f aca="false">IF(F7=0,0,G7/F7)</f>
-        <v>0.215791714279313</v>
+        <v>0.140387071421554</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2764,7 +2764,7 @@
         <v>116</v>
       </c>
       <c r="B8" s="8" t="n">
-        <v>0.18</v>
+        <v>0.21</v>
       </c>
       <c r="C8" s="8" t="n">
         <v>0.18</v>
@@ -2774,19 +2774,19 @@
       </c>
       <c r="E8" s="24" t="n">
         <f aca="false">B8+C8+D8</f>
-        <v>0.41</v>
+        <v>0.44</v>
       </c>
       <c r="F8" s="14" t="n">
         <f aca="false">$B$4*(1-E8)</f>
-        <v>312326.301754286</v>
+        <v>296445.30336</v>
       </c>
       <c r="G8" s="14" t="n">
         <f aca="false">F8-LandedCost!K4</f>
-        <v>75700.1017542858</v>
+        <v>59819.1033600001</v>
       </c>
       <c r="H8" s="24" t="n">
         <f aca="false">IF(F8=0,0,G8/F8)</f>
-        <v>0.242375045998658</v>
+        <v>0.201787994891443</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2794,7 +2794,7 @@
         <v>117</v>
       </c>
       <c r="B9" s="8" t="n">
-        <v>0.15</v>
+        <v>0.17</v>
       </c>
       <c r="C9" s="8" t="n">
         <v>0.05</v>
@@ -2804,19 +2804,19 @@
       </c>
       <c r="E9" s="24" t="n">
         <f aca="false">B9+C9+D9</f>
-        <v>0.23</v>
+        <v>0.25</v>
       </c>
       <c r="F9" s="14" t="n">
         <f aca="false">$B$4*(1-E9)</f>
-        <v>407612.29212</v>
+        <v>397024.959857143</v>
       </c>
       <c r="G9" s="14" t="n">
         <f aca="false">F9-LandedCost!K4</f>
-        <v>170986.09212</v>
+        <v>160398.759857143</v>
       </c>
       <c r="H9" s="24" t="n">
         <f aca="false">IF(F9=0,0,G9/F9)</f>
-        <v>0.419482178102868</v>
+        <v>0.404001702852278</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>